<commit_message>
chore(jdt) mise à jour du jdt pour la journée
</commit_message>
<xml_diff>
--- a/doc/JDT-P_OO.xlsx
+++ b/doc/JDT-P_OO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pi46vew\Documents\GitHub\P_OO-ShootMeUp-\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59696732-849F-44B3-8507-B90E4A6832A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29C56734-DD76-4C6F-818D-EEE02B052121}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$18</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$16</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -354,7 +354,7 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -431,10 +431,6 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
@@ -792,7 +788,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E64"/>
+  <dimension ref="A1:E62"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33" style="1" customWidth="1"/>
@@ -808,10 +804,10 @@
       <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="31" t="s">
+      <c r="B1" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="31"/>
+      <c r="C1" s="30"/>
       <c r="D1" s="19" t="s">
         <v>2</v>
       </c>
@@ -823,10 +819,10 @@
       <c r="A2" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="31" t="s">
+      <c r="B2" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="31"/>
+      <c r="C2" s="30"/>
       <c r="D2" s="19" t="s">
         <v>5</v>
       </c>
@@ -838,10 +834,10 @@
       <c r="A3" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="31" t="s">
+      <c r="B3" s="30" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="31"/>
+      <c r="C3" s="30"/>
       <c r="D3" s="19" t="s">
         <v>8</v>
       </c>
@@ -853,12 +849,12 @@
       <c r="A4" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="32" t="s">
+      <c r="B4" s="31" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="33"/>
-      <c r="D4" s="33"/>
-      <c r="E4" s="34"/>
+      <c r="C4" s="32"/>
+      <c r="D4" s="32"/>
+      <c r="E4" s="33"/>
     </row>
     <row r="5" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -909,7 +905,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
         <v>24</v>
       </c>
@@ -924,99 +920,87 @@
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="7"/>
-      <c r="B9" s="22"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="8"/>
-    </row>
-    <row r="10" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="10"/>
-      <c r="B10" s="23"/>
-      <c r="C10" s="10"/>
-      <c r="D10" s="11"/>
-      <c r="E10" s="10"/>
-    </row>
-    <row r="11" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="12" t="s">
+    <row r="9" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="26"/>
-      <c r="C11" s="27"/>
-      <c r="D11" s="27"/>
-      <c r="E11" s="28"/>
+      <c r="B9" s="25"/>
+      <c r="C9" s="26"/>
+      <c r="D9" s="26"/>
+      <c r="E9" s="27"/>
+    </row>
+    <row r="10" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="4"/>
+      <c r="B10" s="21"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="20"/>
+    </row>
+    <row r="11" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="7"/>
+      <c r="B11" s="23"/>
+      <c r="C11" s="8"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="8"/>
     </row>
     <row r="12" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="4"/>
-      <c r="B12" s="21"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="20"/>
+      <c r="A12" s="7"/>
+      <c r="B12" s="23"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="8"/>
     </row>
     <row r="13" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="7"/>
-      <c r="B13" s="24"/>
+      <c r="B13" s="23"/>
       <c r="C13" s="8"/>
       <c r="D13" s="9"/>
       <c r="E13" s="8"/>
     </row>
-    <row r="14" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="7"/>
+    <row r="14" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="10"/>
       <c r="B14" s="24"/>
-      <c r="C14" s="8"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="8"/>
-    </row>
-    <row r="15" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="7"/>
-      <c r="B15" s="24"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="8"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="10"/>
+    </row>
+    <row r="15" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="25"/>
+      <c r="C15" s="26"/>
+      <c r="D15" s="26"/>
+      <c r="E15" s="27"/>
     </row>
     <row r="16" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="10"/>
-      <c r="B16" s="25"/>
-      <c r="C16" s="10"/>
-      <c r="D16" s="11"/>
-      <c r="E16" s="10"/>
-    </row>
-    <row r="17" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="12" t="s">
-        <v>16</v>
-      </c>
-      <c r="B17" s="26"/>
-      <c r="C17" s="27"/>
-      <c r="D17" s="27"/>
-      <c r="E17" s="28"/>
-    </row>
-    <row r="18" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="29" t="s">
+      <c r="A16" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="B18" s="30"/>
-      <c r="C18" s="13">
-        <f>MROUND(SUM(C6:C16) /60,0.2)</f>
+      <c r="B16" s="29"/>
+      <c r="C16" s="13">
+        <f>MROUND(SUM(C6:C14) /60,0.2)</f>
         <v>3</v>
       </c>
-      <c r="D18" s="14"/>
-      <c r="E18" s="15"/>
-    </row>
-    <row r="19" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="20" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="21" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="22" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="23" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="24" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="25" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="26" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="27" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="1:5" ht="30.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="29" spans="1:5" ht="24.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="30" spans="1:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="31" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="32" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="D16" s="14"/>
+      <c r="E16" s="15"/>
+    </row>
+    <row r="17" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="18" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="19" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="20" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="21" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="22" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="23" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="24" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="25" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="26" ht="30.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="27" ht="24.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="28" ht="21.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="29" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="30" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="31" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="32" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="33" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="34" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="35" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -1046,23 +1030,21 @@
     <row r="59" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="60" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="61" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="62" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="63" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="64" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="62" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="9">
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:E4"/>
-    <mergeCell ref="B6:B10"/>
-    <mergeCell ref="B11:E11"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="B12:B16"/>
-    <mergeCell ref="B17:E17"/>
+    <mergeCell ref="B6:B8"/>
+    <mergeCell ref="B9:E9"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="B10:B14"/>
+    <mergeCell ref="B15:E15"/>
   </mergeCells>
-  <dataValidations disablePrompts="1" count="1">
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B6 C6:C10 B12 C12:C16" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
+  <dataValidations count="1">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B6 C6:C8 B10 C10:C14" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
doc(Rapport de projet) écriture du chapitre "Analyse fonctionnelle" et "Planification Initiale"
</commit_message>
<xml_diff>
--- a/doc/JDT-P_OO.xlsx
+++ b/doc/JDT-P_OO.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pi46vew\Documents\GitHub\P_OO-ShootMeUp-\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29C56734-DD76-4C6F-818D-EEE02B052121}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32776174-4BAE-4575-8CE0-FFC6D2865FC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$16</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$14</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="32">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -130,10 +130,22 @@
     <t>Installation de GitJournal puis rotation vers un journal de travail excel.</t>
   </si>
   <si>
-    <t>Github doc</t>
-  </si>
-  <si>
     <t>Commencé la création d'un gameplan sur paint. Invention du core gameplay et des ennemis/munitions</t>
+  </si>
+  <si>
+    <t>rapport</t>
+  </si>
+  <si>
+    <t>Ecriture des users stories dans le projet Github</t>
+  </si>
+  <si>
+    <t>Ecriture du chapitre Introduction dans le rapport</t>
+  </si>
+  <si>
+    <t>Ecriture du chapitre planification initial dans le rapport</t>
+  </si>
+  <si>
+    <t>github doc P_OO</t>
   </si>
 </sst>
 </file>
@@ -205,7 +217,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -303,32 +315,6 @@
         <color indexed="64"/>
       </right>
       <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="dashed">
         <color indexed="64"/>
       </top>
       <bottom/>
@@ -354,7 +340,7 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -389,14 +375,6 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -422,55 +400,51 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="2" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -788,7 +762,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E62"/>
+  <dimension ref="A1:E60"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33" style="1" customWidth="1"/>
@@ -801,60 +775,60 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="30" t="s">
+      <c r="B1" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="30"/>
-      <c r="D1" s="19" t="s">
+      <c r="C1" s="18"/>
+      <c r="D1" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="17" t="s">
+      <c r="E1" s="15" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="30" t="s">
+      <c r="B2" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="30"/>
-      <c r="D2" s="19" t="s">
+      <c r="C2" s="18"/>
+      <c r="D2" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="17" t="s">
+      <c r="E2" s="15" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="30" t="s">
+      <c r="B3" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="30"/>
-      <c r="D3" s="19" t="s">
+      <c r="C3" s="18"/>
+      <c r="D3" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="16" t="s">
+      <c r="E3" s="14" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="18" t="s">
+      <c r="A4" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="31" t="s">
+      <c r="B4" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="32"/>
-      <c r="D4" s="32"/>
-      <c r="E4" s="33"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="21"/>
     </row>
     <row r="5" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -877,7 +851,7 @@
       <c r="A6" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="21">
+      <c r="B6" s="22">
         <v>45894</v>
       </c>
       <c r="C6" s="5">
@@ -886,105 +860,119 @@
       <c r="D6" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="E6" s="20" t="s">
-        <v>26</v>
+      <c r="E6" s="30" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B7" s="22"/>
+      <c r="B7" s="23"/>
       <c r="C7" s="8">
         <v>45</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="E7" s="20" t="s">
         <v>26</v>
+      </c>
+      <c r="E7" s="30" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="B8" s="22"/>
+      <c r="B8" s="23"/>
       <c r="C8" s="8">
         <v>45</v>
       </c>
       <c r="D8" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="E8" s="20" t="s">
-        <v>26</v>
+      <c r="E8" s="30" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="25"/>
-      <c r="C9" s="26"/>
-      <c r="D9" s="26"/>
-      <c r="E9" s="27"/>
+      <c r="B9" s="24"/>
+      <c r="C9" s="25"/>
+      <c r="D9" s="25"/>
+      <c r="E9" s="26"/>
     </row>
-    <row r="10" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="4"/>
-      <c r="B10" s="21"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="20"/>
+    <row r="10" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" s="22">
+        <v>46269</v>
+      </c>
+      <c r="C10" s="5">
+        <v>45</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="E10" s="30" t="s">
+        <v>31</v>
+      </c>
     </row>
-    <row r="11" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="7"/>
-      <c r="B11" s="23"/>
-      <c r="C11" s="8"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="8"/>
+    <row r="11" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11" s="29"/>
+      <c r="C11" s="8">
+        <v>120</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="E11" s="30" t="s">
+        <v>31</v>
+      </c>
     </row>
-    <row r="12" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="7"/>
-      <c r="B12" s="23"/>
-      <c r="C12" s="8"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="8"/>
+    <row r="12" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" s="29"/>
+      <c r="C12" s="8">
+        <v>15</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="E12" s="30" t="s">
+        <v>31</v>
+      </c>
     </row>
-    <row r="13" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="7"/>
-      <c r="B13" s="23"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="8"/>
+    <row r="13" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13" s="24"/>
+      <c r="C13" s="25"/>
+      <c r="D13" s="25"/>
+      <c r="E13" s="26"/>
     </row>
     <row r="14" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="10"/>
-      <c r="B14" s="24"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="11"/>
-      <c r="E14" s="10"/>
+      <c r="A14" s="27" t="s">
+        <v>17</v>
+      </c>
+      <c r="B14" s="28"/>
+      <c r="C14" s="11">
+        <f>MROUND(SUM(C6:C12) /60,0.2)</f>
+        <v>6</v>
+      </c>
+      <c r="D14" s="12"/>
+      <c r="E14" s="13"/>
     </row>
-    <row r="15" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="12" t="s">
-        <v>16</v>
-      </c>
-      <c r="B15" s="25"/>
-      <c r="C15" s="26"/>
-      <c r="D15" s="26"/>
-      <c r="E15" s="27"/>
-    </row>
-    <row r="16" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="28" t="s">
-        <v>17</v>
-      </c>
-      <c r="B16" s="29"/>
-      <c r="C16" s="13">
-        <f>MROUND(SUM(C6:C14) /60,0.2)</f>
-        <v>3</v>
-      </c>
-      <c r="D16" s="14"/>
-      <c r="E16" s="15"/>
-    </row>
+    <row r="15" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="18" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="19" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -992,11 +980,11 @@
     <row r="21" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="22" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="23" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="24" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="25" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="26" ht="30.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="27" ht="24.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="28" ht="21.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="24" ht="30.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="25" ht="24.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="26" ht="21.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="27" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="28" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="29" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="30" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="31" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -1028,34 +1016,40 @@
     <row r="57" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="58" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="59" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="60" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="61" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="62" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="60" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="9">
+    <mergeCell ref="B9:E9"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="B10:B12"/>
+    <mergeCell ref="B13:E13"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:E4"/>
     <mergeCell ref="B6:B8"/>
-    <mergeCell ref="B9:E9"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="B10:B14"/>
-    <mergeCell ref="B15:E15"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B6 C6:C8 B10 C10:C14" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B6 C6:C8 B10 C10:C12" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="E6" r:id="rId1" xr:uid="{A9036453-85A7-4AAB-A068-2C8808FAA421}"/>
+    <hyperlink ref="E7" r:id="rId2" xr:uid="{8D7EF9C7-935B-472B-8557-2C6033A13EF1}"/>
+    <hyperlink ref="E8" r:id="rId3" xr:uid="{275F9030-7E94-44FA-A7D6-B4F673D98F13}"/>
+    <hyperlink ref="E10" r:id="rId4" xr:uid="{966E8E29-D905-4447-A9DB-EB329198F989}"/>
+    <hyperlink ref="E11" r:id="rId5" xr:uid="{6C90BBFF-ACB5-4E0E-88DD-D90956D88243}"/>
+    <hyperlink ref="E12" r:id="rId6" xr:uid="{E58BEBDD-E502-4AF4-80D2-67E709673300}"/>
+  </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="43" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="43" orientation="portrait" r:id="rId7"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Etml_font,Normal"&amp;22ETML&amp;R&amp;G</oddHeader>
     <oddFooter>&amp;L&amp;14&amp;D&amp;R&amp;14Journal</oddFooter>
   </headerFooter>
-  <legacyDrawingHF r:id="rId2"/>
+  <legacyDrawingHF r:id="rId8"/>
 </worksheet>
 </file>
 
@@ -1072,15 +1066,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010051C931FEC57CD24D841BB655C8BA0DFF" ma:contentTypeVersion="14" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="f47e485f4ad8d247f3dfedaee1362e95">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3eb094ff-ec8d-44d8-be06-94ad3ec8832a" xmlns:ns3="4356f79f-5386-4bda-9d92-82d8bd7b074e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="da34bf24383b1ce13aa9c82f6b8627bb" ns2:_="" ns3:_="">
     <xsd:import namespace="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
@@ -1293,6 +1278,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
   <ds:schemaRefs>
@@ -1305,14 +1299,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5A40649F-4D7C-4B62-9A51-E0A7D9450EFE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1329,4 +1315,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
fix(JDT, Rapport) corriger des détails du JDT et rapport
</commit_message>
<xml_diff>
--- a/doc/JDT-P_OO.xlsx
+++ b/doc/JDT-P_OO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pi46vew\Documents\GitHub\P_OO-ShootMeUp-\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32776174-4BAE-4575-8CE0-FFC6D2865FC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{671E4532-A50B-41EF-9E91-FCE3D5146739}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="33">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -51,9 +51,6 @@
   </si>
   <si>
     <t>Classe ou Groupe</t>
-  </si>
-  <si>
-    <t>GRP1D</t>
   </si>
   <si>
     <t>Experts </t>
@@ -146,6 +143,12 @@
   </si>
   <si>
     <t>github doc P_OO</t>
+  </si>
+  <si>
+    <t>MID2B</t>
+  </si>
+  <si>
+    <t>projet P_OO</t>
   </si>
 </sst>
 </file>
@@ -786,7 +789,7 @@
         <v>2</v>
       </c>
       <c r="E1" s="15" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -794,37 +797,37 @@
         <v>3</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>4</v>
+        <v>31</v>
       </c>
       <c r="C2" s="18"/>
       <c r="D2" s="17" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="15" t="s">
         <v>5</v>
-      </c>
-      <c r="E2" s="15" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="16" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C3" s="18"/>
       <c r="D3" s="17" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="16" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C4" s="20"/>
       <c r="D4" s="20"/>
@@ -832,24 +835,24 @@
     </row>
     <row r="5" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="E5" s="2" t="s">
         <v>13</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B6" s="22">
         <v>45894</v>
@@ -858,45 +861,45 @@
         <v>90</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E6" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B7" s="23"/>
       <c r="C7" s="8">
         <v>45</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E7" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B8" s="23"/>
       <c r="C8" s="8">
         <v>45</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E8" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B9" s="24"/>
       <c r="C9" s="25"/>
@@ -905,7 +908,7 @@
     </row>
     <row r="10" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B10" s="22">
         <v>46269</v>
@@ -914,45 +917,45 @@
         <v>45</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E10" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B11" s="29"/>
       <c r="C11" s="8">
         <v>120</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E11" s="30" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B12" s="29"/>
       <c r="C12" s="8">
         <v>15</v>
       </c>
       <c r="D12" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="E12" s="30" t="s">
         <v>30</v>
-      </c>
-      <c r="E12" s="30" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B13" s="24"/>
       <c r="C13" s="25"/>
@@ -961,7 +964,7 @@
     </row>
     <row r="14" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="27" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B14" s="28"/>
       <c r="C14" s="11">
@@ -1035,12 +1038,12 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="E6" r:id="rId1" xr:uid="{A9036453-85A7-4AAB-A068-2C8808FAA421}"/>
-    <hyperlink ref="E7" r:id="rId2" xr:uid="{8D7EF9C7-935B-472B-8557-2C6033A13EF1}"/>
-    <hyperlink ref="E8" r:id="rId3" xr:uid="{275F9030-7E94-44FA-A7D6-B4F673D98F13}"/>
-    <hyperlink ref="E10" r:id="rId4" xr:uid="{966E8E29-D905-4447-A9DB-EB329198F989}"/>
-    <hyperlink ref="E11" r:id="rId5" xr:uid="{6C90BBFF-ACB5-4E0E-88DD-D90956D88243}"/>
-    <hyperlink ref="E12" r:id="rId6" xr:uid="{E58BEBDD-E502-4AF4-80D2-67E709673300}"/>
+    <hyperlink ref="E8" r:id="rId1" xr:uid="{275F9030-7E94-44FA-A7D6-B4F673D98F13}"/>
+    <hyperlink ref="E10" r:id="rId2" xr:uid="{966E8E29-D905-4447-A9DB-EB329198F989}"/>
+    <hyperlink ref="E7" r:id="rId3" xr:uid="{0B7914AF-AD3B-41DB-B0A0-11394DCCB3C2}"/>
+    <hyperlink ref="E6" r:id="rId4" xr:uid="{E03124A8-1F2B-48D7-B6CA-5B37E7D01F3C}"/>
+    <hyperlink ref="E12" r:id="rId5" xr:uid="{335585FC-0447-4C05-B123-6F458771495A}"/>
+    <hyperlink ref="E11" r:id="rId6" xr:uid="{3E1620A4-D69C-41AE-9BF1-38B41484B637}"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
@@ -1290,10 +1293,16 @@
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
   <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="4356f79f-5386-4bda-9d92-82d8bd7b074e"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="4356f79f-5386-4bda-9d92-82d8bd7b074e"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
     <ds:schemaRef ds:uri="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
chore(base) ajout de la base de code inspiré de l'exercice Drone
</commit_message>
<xml_diff>
--- a/doc/JDT-P_OO.xlsx
+++ b/doc/JDT-P_OO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pi46vew\Documents\GitHub\P_OO-ShootMeUp-\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{671E4532-A50B-41EF-9E91-FCE3D5146739}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CE2312F-FB3D-4153-8A87-A09F0E9353AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$14</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$32</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="39">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -149,6 +149,24 @@
   </si>
   <si>
     <t>projet P_OO</t>
+  </si>
+  <si>
+    <t>user stories</t>
+  </si>
+  <si>
+    <t>Ecriture des users stories 8,9,5,6,10 dans le projet Github</t>
+  </si>
+  <si>
+    <t>Découverte du code "Base"</t>
+  </si>
+  <si>
+    <t>Prise de connaissance du code Base</t>
+  </si>
+  <si>
+    <t>Correction du rapport</t>
+  </si>
+  <si>
+    <t>Correction de quelque faute relevé par le prof dans mon rapport et user stories</t>
   </si>
 </sst>
 </file>
@@ -220,7 +238,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -229,16 +247,14 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
+      <left/>
       <right style="medium">
         <color indexed="64"/>
       </right>
       <top style="medium">
         <color indexed="64"/>
       </top>
-      <bottom style="dashed">
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -247,15 +263,107 @@
       <left style="medium">
         <color indexed="64"/>
       </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="dashed">
+      <top style="medium">
         <color indexed="64"/>
       </top>
-      <bottom style="dashed">
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -264,62 +372,6 @@
       <top style="medium">
         <color indexed="64"/>
       </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -327,9 +379,7 @@
       <left style="medium">
         <color indexed="64"/>
       </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
+      <right/>
       <top/>
       <bottom/>
       <diagonal/>
@@ -343,111 +393,172 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -765,7 +876,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E60"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33" style="1" customWidth="1"/>
@@ -778,220 +889,277 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18" t="s">
+      <c r="B1" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="18"/>
-      <c r="D1" s="17" t="s">
+      <c r="C1" s="14"/>
+      <c r="D1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="E1" s="6" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="18"/>
-      <c r="D2" s="17" t="s">
+      <c r="C2" s="14"/>
+      <c r="D2" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="15" t="s">
+      <c r="E2" s="6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="16" t="s">
+    <row r="3" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="18"/>
-      <c r="D3" s="17" t="s">
+      <c r="C3" s="14"/>
+      <c r="D3" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="14" t="s">
+      <c r="E3" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="16" t="s">
+      <c r="A4" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="20"/>
-      <c r="D4" s="20"/>
-      <c r="E4" s="21"/>
-    </row>
-    <row r="5" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
+      <c r="C4" s="23"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="24"/>
+    </row>
+    <row r="5" spans="1:5" s="26" customFormat="1" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="25" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="4" t="s">
+    <row r="6" spans="1:5" s="26" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="22">
+      <c r="B6" s="12">
         <v>45894</v>
       </c>
-      <c r="C6" s="5">
+      <c r="C6" s="30">
         <v>90</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="E6" s="30" t="s">
+      <c r="E6" s="39" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="7" t="s">
+    <row r="7" spans="1:5" s="26" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="23"/>
-      <c r="C7" s="8">
+      <c r="B7" s="15"/>
+      <c r="C7" s="9">
         <v>45</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="37" t="s">
         <v>25</v>
       </c>
-      <c r="E7" s="30" t="s">
+      <c r="E7" s="40" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="7" t="s">
+    <row r="8" spans="1:5" s="26" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="23"/>
-      <c r="C8" s="8">
+      <c r="B8" s="29"/>
+      <c r="C8" s="31">
         <v>45</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="D8" s="38" t="s">
         <v>24</v>
       </c>
-      <c r="E8" s="30" t="s">
+      <c r="E8" s="41" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="10" t="s">
+    <row r="9" spans="1:5" s="26" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="24"/>
-      <c r="C9" s="25"/>
-      <c r="D9" s="25"/>
-      <c r="E9" s="26"/>
-    </row>
-    <row r="10" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="4" t="s">
+      <c r="B9" s="35"/>
+      <c r="C9" s="42">
+        <f>SUM(C6:C8)</f>
+        <v>180</v>
+      </c>
+      <c r="D9" s="35"/>
+      <c r="E9" s="35"/>
+    </row>
+    <row r="10" spans="1:5" s="26" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="B10" s="22">
+      <c r="B10" s="32">
         <v>46269</v>
       </c>
-      <c r="C10" s="5">
+      <c r="C10" s="30">
         <v>45</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D10" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="E10" s="30" t="s">
+      <c r="E10" s="28" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="4" t="s">
+    <row r="11" spans="1:5" s="26" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="29"/>
-      <c r="C11" s="8">
+      <c r="B11" s="33"/>
+      <c r="C11" s="9">
         <v>120</v>
       </c>
-      <c r="D11" s="9" t="s">
+      <c r="D11" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="E11" s="30" t="s">
+      <c r="E11" s="28" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="4" t="s">
+    <row r="12" spans="1:5" s="26" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="B12" s="29"/>
-      <c r="C12" s="8">
+      <c r="B12" s="34"/>
+      <c r="C12" s="31">
         <v>15</v>
       </c>
-      <c r="D12" s="9" t="s">
+      <c r="D12" s="27" t="s">
         <v>29</v>
       </c>
-      <c r="E12" s="30" t="s">
+      <c r="E12" s="28" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="10" t="s">
+    <row r="13" spans="1:5" s="26" customFormat="1" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="24"/>
-      <c r="C13" s="25"/>
-      <c r="D13" s="25"/>
-      <c r="E13" s="26"/>
-    </row>
-    <row r="14" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="27" t="s">
+      <c r="B13" s="35"/>
+      <c r="C13" s="42">
+        <f>SUM(C10:C12)</f>
+        <v>180</v>
+      </c>
+      <c r="D13" s="35"/>
+      <c r="E13" s="35"/>
+    </row>
+    <row r="14" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="B14" s="12">
+        <v>46276</v>
+      </c>
+      <c r="C14" s="30">
+        <v>60</v>
+      </c>
+      <c r="D14" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="E14" s="39" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" s="26" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="B15" s="13"/>
+      <c r="C15" s="46">
+        <v>20</v>
+      </c>
+      <c r="D15" s="26" t="s">
+        <v>38</v>
+      </c>
+      <c r="E15" s="40"/>
+    </row>
+    <row r="16" spans="1:5" s="26" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16" s="13"/>
+      <c r="C16" s="9">
+        <v>10</v>
+      </c>
+      <c r="D16" s="45" t="s">
+        <v>36</v>
+      </c>
+      <c r="E16" s="40"/>
+    </row>
+    <row r="17" spans="1:5" s="26" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="B17" s="35"/>
+      <c r="C17" s="42">
+        <f>SUM(C14:C16)</f>
+        <v>90</v>
+      </c>
+      <c r="D17" s="35"/>
+      <c r="E17" s="35"/>
+    </row>
+    <row r="18" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="19" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="20" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="21" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="22" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="23" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="24" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="25" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="27" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="28" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="29" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="30" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="31" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="32" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="28"/>
-      <c r="C14" s="11">
-        <f>MROUND(SUM(C6:C12) /60,0.2)</f>
-        <v>6</v>
-      </c>
-      <c r="D14" s="12"/>
-      <c r="E14" s="13"/>
-    </row>
-    <row r="15" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="16" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="17" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="18" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="19" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="20" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="21" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="22" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="23" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="24" ht="30.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="25" ht="24.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="26" ht="21.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="27" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="28" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="29" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="30" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="31" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="32" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="B32" s="11"/>
+      <c r="C32" s="2">
+        <f>MROUND(SUM(C6:C31) /60,0.2)</f>
+        <v>15</v>
+      </c>
+      <c r="D32" s="3"/>
+      <c r="E32" s="4"/>
+    </row>
     <row r="33" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="34" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="35" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -1009,23 +1177,12 @@
     <row r="47" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="48" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="49" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="50" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="51" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="52" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="53" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="54" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="55" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="56" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="57" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="58" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="59" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="60" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="50" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="B9:E9"/>
-    <mergeCell ref="A14:B14"/>
+  <mergeCells count="8">
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="A32:B32"/>
     <mergeCell ref="B10:B12"/>
-    <mergeCell ref="B13:E13"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
@@ -1033,7 +1190,7 @@
     <mergeCell ref="B6:B8"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B6 C6:C8 B10 C10:C12" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B6 C6:C8 B10 C10:C12 C16 B14:C14" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -1044,15 +1201,16 @@
     <hyperlink ref="E6" r:id="rId4" xr:uid="{E03124A8-1F2B-48D7-B6CA-5B37E7D01F3C}"/>
     <hyperlink ref="E12" r:id="rId5" xr:uid="{335585FC-0447-4C05-B123-6F458771495A}"/>
     <hyperlink ref="E11" r:id="rId6" xr:uid="{3E1620A4-D69C-41AE-9BF1-38B41484B637}"/>
+    <hyperlink ref="E14" r:id="rId7" xr:uid="{8ED2937A-5238-4FAF-83F2-4DF75BCBD4C3}"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="43" orientation="portrait" r:id="rId7"/>
+  <pageSetup paperSize="9" scale="43" orientation="portrait" r:id="rId8"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Etml_font,Normal"&amp;22ETML&amp;R&amp;G</oddHeader>
     <oddFooter>&amp;L&amp;14&amp;D&amp;R&amp;14Journal</oddFooter>
   </headerFooter>
-  <legacyDrawingHF r:id="rId8"/>
+  <legacyDrawingHF r:id="rId9"/>
 </worksheet>
 </file>
 
@@ -1069,6 +1227,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010051C931FEC57CD24D841BB655C8BA0DFF" ma:contentTypeVersion="14" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="f47e485f4ad8d247f3dfedaee1362e95">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3eb094ff-ec8d-44d8-be06-94ad3ec8832a" xmlns:ns3="4356f79f-5386-4bda-9d92-82d8bd7b074e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="da34bf24383b1ce13aa9c82f6b8627bb" ns2:_="" ns3:_="">
     <xsd:import namespace="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
@@ -1281,15 +1448,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
   <ds:schemaRefs>
@@ -1308,6 +1466,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5A40649F-4D7C-4B62-9A51-E0A7D9450EFE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1324,12 +1490,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat(Déplacement) finis le déplacement du joueur de manière orthogonal et diagonal.
</commit_message>
<xml_diff>
--- a/doc/JDT-P_OO.xlsx
+++ b/doc/JDT-P_OO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pi46vew\Documents\GitHub\P_OO-ShootMeUp-\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CE2312F-FB3D-4153-8A87-A09F0E9353AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4300F201-F918-4C88-9E1C-D18A4A481B38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="39">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -238,7 +238,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -384,6 +384,17 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -393,7 +404,7 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -423,50 +434,123 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
@@ -476,89 +560,56 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -892,10 +943,10 @@
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="14"/>
+      <c r="C1" s="40"/>
       <c r="D1" s="8" t="s">
         <v>2</v>
       </c>
@@ -907,10 +958,10 @@
       <c r="A2" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="40" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="14"/>
+      <c r="C2" s="40"/>
       <c r="D2" s="8" t="s">
         <v>4</v>
       </c>
@@ -922,10 +973,10 @@
       <c r="A3" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="14"/>
+      <c r="C3" s="40"/>
       <c r="D3" s="8" t="s">
         <v>7</v>
       </c>
@@ -934,212 +985,253 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="21" t="s">
+      <c r="A4" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="22" t="s">
+      <c r="B4" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="23"/>
-      <c r="D4" s="23"/>
-      <c r="E4" s="24"/>
-    </row>
-    <row r="5" spans="1:5" s="26" customFormat="1" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="25" t="s">
+      <c r="C4" s="42"/>
+      <c r="D4" s="42"/>
+      <c r="E4" s="43"/>
+    </row>
+    <row r="5" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="25" t="s">
+      <c r="B5" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="25" t="s">
+      <c r="C5" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="25" t="s">
+      <c r="D5" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="25" t="s">
+      <c r="E5" s="16" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:5" s="26" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="17" t="s">
+    <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="12">
+      <c r="B6" s="33">
         <v>45894</v>
       </c>
-      <c r="C6" s="30">
+      <c r="C6" s="20">
         <v>90</v>
       </c>
-      <c r="D6" s="36" t="s">
+      <c r="D6" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="E6" s="39" t="s">
+      <c r="E6" s="25" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:5" s="26" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="18" t="s">
+    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="15"/>
+      <c r="B7" s="44"/>
       <c r="C7" s="9">
         <v>45</v>
       </c>
-      <c r="D7" s="37" t="s">
+      <c r="D7" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="E7" s="40" t="s">
+      <c r="E7" s="26" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:5" s="26" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="19" t="s">
+    <row r="8" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="29"/>
-      <c r="C8" s="31">
+      <c r="B8" s="45"/>
+      <c r="C8" s="19">
         <v>45</v>
       </c>
-      <c r="D8" s="38" t="s">
+      <c r="D8" s="24" t="s">
         <v>24</v>
       </c>
-      <c r="E8" s="41" t="s">
+      <c r="E8" s="27" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:5" s="26" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="20" t="s">
+    <row r="9" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="35"/>
-      <c r="C9" s="42">
+      <c r="B9" s="21"/>
+      <c r="C9" s="28">
         <f>SUM(C6:C8)</f>
         <v>180</v>
       </c>
-      <c r="D9" s="35"/>
-      <c r="E9" s="35"/>
-    </row>
-    <row r="10" spans="1:5" s="26" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="17" t="s">
+      <c r="D9" s="21"/>
+      <c r="E9" s="21"/>
+    </row>
+    <row r="10" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="B10" s="32">
+      <c r="B10" s="37">
         <v>46269</v>
       </c>
-      <c r="C10" s="30">
+      <c r="C10" s="20">
         <v>45</v>
       </c>
-      <c r="D10" s="27" t="s">
+      <c r="D10" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="E10" s="28" t="s">
+      <c r="E10" s="18" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:5" s="26" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="18" t="s">
+    <row r="11" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="33"/>
+      <c r="B11" s="38"/>
       <c r="C11" s="9">
         <v>120</v>
       </c>
-      <c r="D11" s="27" t="s">
+      <c r="D11" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="E11" s="28" t="s">
+      <c r="E11" s="18" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="12" spans="1:5" s="26" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="19" t="s">
+    <row r="12" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="B12" s="34"/>
-      <c r="C12" s="31">
+      <c r="B12" s="39"/>
+      <c r="C12" s="19">
         <v>15</v>
       </c>
-      <c r="D12" s="27" t="s">
+      <c r="D12" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="E12" s="28" t="s">
+      <c r="E12" s="18" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="1:5" s="26" customFormat="1" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="16" t="s">
+    <row r="13" spans="1:5" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="35"/>
-      <c r="C13" s="42">
+      <c r="B13" s="21"/>
+      <c r="C13" s="28">
         <f>SUM(C10:C12)</f>
         <v>180</v>
       </c>
-      <c r="D13" s="35"/>
-      <c r="E13" s="35"/>
-    </row>
-    <row r="14" spans="1:5" s="26" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="17" t="s">
+      <c r="D13" s="21"/>
+      <c r="E13" s="21"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="B14" s="12">
+      <c r="B14" s="33">
         <v>46276</v>
       </c>
-      <c r="C14" s="30">
+      <c r="C14" s="20">
         <v>60</v>
       </c>
-      <c r="D14" s="44" t="s">
+      <c r="D14" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="E14" s="39" t="s">
+      <c r="E14" s="25" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="15" spans="1:5" s="26" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="43" t="s">
+    <row r="15" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="29" t="s">
         <v>37</v>
       </c>
-      <c r="B15" s="13"/>
-      <c r="C15" s="46">
+      <c r="B15" s="34"/>
+      <c r="C15" s="32">
         <v>20</v>
       </c>
-      <c r="D15" s="26" t="s">
+      <c r="D15" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E15" s="40"/>
-    </row>
-    <row r="16" spans="1:5" s="26" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="18" t="s">
+      <c r="E15" s="26"/>
+    </row>
+    <row r="16" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="B16" s="13"/>
+      <c r="B16" s="34"/>
       <c r="C16" s="9">
         <v>10</v>
       </c>
-      <c r="D16" s="45" t="s">
+      <c r="D16" s="31" t="s">
         <v>36</v>
       </c>
-      <c r="E16" s="40"/>
-    </row>
-    <row r="17" spans="1:5" s="26" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="16" t="s">
+      <c r="E16" s="26"/>
+    </row>
+    <row r="17" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="35"/>
-      <c r="C17" s="42">
+      <c r="B17" s="55"/>
+      <c r="C17" s="28">
         <f>SUM(C14:C16)</f>
         <v>90</v>
       </c>
-      <c r="D17" s="35"/>
-      <c r="E17" s="35"/>
-    </row>
-    <row r="18" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="19" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="20" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="21" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="22" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="23" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="D17" s="21"/>
+      <c r="E17" s="21"/>
+    </row>
+    <row r="18" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="46"/>
+      <c r="B18" s="33">
+        <v>46283</v>
+      </c>
+      <c r="C18" s="48"/>
+      <c r="D18" s="22"/>
+      <c r="E18" s="25"/>
+    </row>
+    <row r="19" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="29"/>
+      <c r="B19" s="34"/>
+      <c r="C19" s="49"/>
+      <c r="D19" s="51"/>
+      <c r="E19" s="26"/>
+    </row>
+    <row r="20" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="47"/>
+      <c r="B20" s="34"/>
+      <c r="C20" s="50"/>
+      <c r="D20" s="23"/>
+      <c r="E20" s="26"/>
+    </row>
+    <row r="21" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="34"/>
+      <c r="C21" s="53"/>
+      <c r="D21" s="51"/>
+      <c r="E21" s="51"/>
+    </row>
+    <row r="22" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="57"/>
+      <c r="C22" s="54"/>
+      <c r="D22" s="52"/>
+      <c r="E22" s="52"/>
+    </row>
+    <row r="23" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B23" s="56"/>
+      <c r="C23" s="28">
+        <f>SUM(C18:C20)</f>
+        <v>0</v>
+      </c>
+      <c r="D23" s="21"/>
+      <c r="E23" s="21"/>
+    </row>
     <row r="24" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="25" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="26" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -1149,10 +1241,10 @@
     <row r="30" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="31" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="32" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="10" t="s">
+      <c r="A32" s="35" t="s">
         <v>16</v>
       </c>
-      <c r="B32" s="11"/>
+      <c r="B32" s="36"/>
       <c r="C32" s="2">
         <f>MROUND(SUM(C6:C31) /60,0.2)</f>
         <v>15</v>
@@ -1179,7 +1271,7 @@
     <row r="49" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="50" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="B14:B16"/>
     <mergeCell ref="A32:B32"/>
     <mergeCell ref="B10:B12"/>
@@ -1188,9 +1280,10 @@
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:E4"/>
     <mergeCell ref="B6:B8"/>
+    <mergeCell ref="B18:B22"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B6 C6:C8 B10 C10:C12 C16 B14:C14" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B6 C6:C8 B10 C10:C12 C16 B14:C14 C20 B18:C18" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -1227,15 +1320,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010051C931FEC57CD24D841BB655C8BA0DFF" ma:contentTypeVersion="14" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="f47e485f4ad8d247f3dfedaee1362e95">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3eb094ff-ec8d-44d8-be06-94ad3ec8832a" xmlns:ns3="4356f79f-5386-4bda-9d92-82d8bd7b074e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="da34bf24383b1ce13aa9c82f6b8627bb" ns2:_="" ns3:_="">
     <xsd:import namespace="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
@@ -1448,6 +1532,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
   <ds:schemaRefs>
@@ -1466,14 +1559,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5A40649F-4D7C-4B62-9A51-E0A7D9450EFE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1490,4 +1575,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
refactor(Déplacement) passage d'une liste de char à une liste de string
</commit_message>
<xml_diff>
--- a/doc/JDT-P_OO.xlsx
+++ b/doc/JDT-P_OO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pi46vew\Documents\GitHub\P_OO-ShootMeUp-\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4300F201-F918-4C88-9E1C-D18A4A481B38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEC4791E-1438-4C9B-8845-5B59A8A51778}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="41">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -167,6 +167,12 @@
   </si>
   <si>
     <t>Correction de quelque faute relevé par le prof dans mon rapport et user stories</t>
+  </si>
+  <si>
+    <t>Déplacement</t>
+  </si>
+  <si>
+    <t>Ajout d'un déplacement orthogonale et diagonale dans le jeu pour le joueur. (User Story num 1)</t>
   </si>
 </sst>
 </file>
@@ -1186,12 +1192,18 @@
       <c r="E17" s="21"/>
     </row>
     <row r="18" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="46"/>
+      <c r="A18" s="46" t="s">
+        <v>39</v>
+      </c>
       <c r="B18" s="33">
         <v>46283</v>
       </c>
-      <c r="C18" s="48"/>
-      <c r="D18" s="22"/>
+      <c r="C18" s="48">
+        <v>50</v>
+      </c>
+      <c r="D18" s="22" t="s">
+        <v>40</v>
+      </c>
       <c r="E18" s="25"/>
     </row>
     <row r="19" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1227,7 +1239,7 @@
       <c r="B23" s="56"/>
       <c r="C23" s="28">
         <f>SUM(C18:C20)</f>
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="D23" s="21"/>
       <c r="E23" s="21"/>
@@ -1247,7 +1259,7 @@
       <c r="B32" s="36"/>
       <c r="C32" s="2">
         <f>MROUND(SUM(C6:C31) /60,0.2)</f>
-        <v>15</v>
+        <v>16.600000000000001</v>
       </c>
       <c r="D32" s="3"/>
       <c r="E32" s="4"/>

</xml_diff>

<commit_message>
feat(attaque burger) instanciation d'un burger sur la souris
</commit_message>
<xml_diff>
--- a/doc/JDT-P_OO.xlsx
+++ b/doc/JDT-P_OO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pi46vew\Documents\GitHub\P_OO-ShootMeUp-\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEC4791E-1438-4C9B-8845-5B59A8A51778}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3974447-B039-4663-BC36-B49E4E67D272}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="44">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -172,7 +172,16 @@
     <t>Déplacement</t>
   </si>
   <si>
-    <t>Ajout d'un déplacement orthogonale et diagonale dans le jeu pour le joueur. (User Story num 1)</t>
+    <t>Attaque burger</t>
+  </si>
+  <si>
+    <t>Ajout d'un déplacement orthogonale et diagonale pour le joueur. (User Story num 1)</t>
+  </si>
+  <si>
+    <t>Ajout d'un burger sur la carte (User Story num 2)</t>
+  </si>
+  <si>
+    <t>Détection des touches de la souris (User Story num 2)</t>
   </si>
 </sst>
 </file>
@@ -1202,22 +1211,34 @@
         <v>50</v>
       </c>
       <c r="D18" s="22" t="s">
+        <v>41</v>
+      </c>
+      <c r="E18" s="25"/>
+    </row>
+    <row r="19" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="E18" s="25"/>
-    </row>
-    <row r="19" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="29"/>
       <c r="B19" s="34"/>
-      <c r="C19" s="49"/>
-      <c r="D19" s="51"/>
+      <c r="C19" s="49">
+        <v>40</v>
+      </c>
+      <c r="D19" s="51" t="s">
+        <v>42</v>
+      </c>
       <c r="E19" s="26"/>
     </row>
     <row r="20" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="47"/>
+      <c r="A20" s="47" t="s">
+        <v>40</v>
+      </c>
       <c r="B20" s="34"/>
-      <c r="C20" s="50"/>
-      <c r="D20" s="23"/>
+      <c r="C20" s="50">
+        <v>30</v>
+      </c>
+      <c r="D20" s="23" t="s">
+        <v>43</v>
+      </c>
       <c r="E20" s="26"/>
     </row>
     <row r="21" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1239,7 +1260,7 @@
       <c r="B23" s="56"/>
       <c r="C23" s="28">
         <f>SUM(C18:C20)</f>
-        <v>50</v>
+        <v>120</v>
       </c>
       <c r="D23" s="21"/>
       <c r="E23" s="21"/>
@@ -1259,7 +1280,7 @@
       <c r="B32" s="36"/>
       <c r="C32" s="2">
         <f>MROUND(SUM(C6:C31) /60,0.2)</f>
-        <v>16.600000000000001</v>
+        <v>19</v>
       </c>
       <c r="D32" s="3"/>
       <c r="E32" s="4"/>

</xml_diff>

<commit_message>
chore(JDT) mis à jour du JDT
</commit_message>
<xml_diff>
--- a/doc/JDT-P_OO.xlsx
+++ b/doc/JDT-P_OO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pi46vew\Documents\GitHub\P_OO-ShootMeUp-\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3974447-B039-4663-BC36-B49E4E67D272}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36EB7A0E-A7FB-44E6-9374-C70E22551C5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="45">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -182,6 +182,9 @@
   </si>
   <si>
     <t>Détection des touches de la souris (User Story num 2)</t>
+  </si>
+  <si>
+    <t>Instantiation du burger sur la carte lors du clique mais pas réussi à ajouter la trajectoire (User Story num 2)</t>
   </si>
 </sst>
 </file>
@@ -253,7 +256,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -399,17 +402,6 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -419,7 +411,7 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -605,25 +597,8 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -1192,7 +1167,7 @@
       <c r="A17" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="55"/>
+      <c r="B17" s="52"/>
       <c r="C17" s="28">
         <f>SUM(C14:C16)</f>
         <v>90</v>
@@ -1241,30 +1216,32 @@
       </c>
       <c r="E20" s="26"/>
     </row>
-    <row r="21" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="47" t="s">
+        <v>40</v>
+      </c>
       <c r="B21" s="34"/>
-      <c r="C21" s="53"/>
-      <c r="D21" s="51"/>
+      <c r="C21" s="49">
+        <v>60</v>
+      </c>
+      <c r="D21" s="51" t="s">
+        <v>44</v>
+      </c>
       <c r="E21" s="51"/>
     </row>
     <row r="22" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="57"/>
-      <c r="C22" s="54"/>
-      <c r="D22" s="52"/>
-      <c r="E22" s="52"/>
-    </row>
-    <row r="23" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="10" t="s">
+      <c r="A22" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B23" s="56"/>
-      <c r="C23" s="28">
-        <f>SUM(C18:C20)</f>
-        <v>120</v>
-      </c>
-      <c r="D23" s="21"/>
-      <c r="E23" s="21"/>
-    </row>
+      <c r="B22" s="21"/>
+      <c r="C22" s="28">
+        <f>SUM(C18:C21)</f>
+        <v>180</v>
+      </c>
+      <c r="D22" s="21"/>
+      <c r="E22" s="21"/>
+    </row>
+    <row r="23" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="24" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="25" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="26" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -1280,7 +1257,7 @@
       <c r="B32" s="36"/>
       <c r="C32" s="2">
         <f>MROUND(SUM(C6:C31) /60,0.2)</f>
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D32" s="3"/>
       <c r="E32" s="4"/>
@@ -1313,7 +1290,7 @@
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:E4"/>
     <mergeCell ref="B6:B8"/>
-    <mergeCell ref="B18:B22"/>
+    <mergeCell ref="B18:B21"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B6 C6:C8 B10 C10:C12 C16 B14:C14 C20 B18:C18" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">

</xml_diff>

<commit_message>
feat(attaque burger) les burgeurs vont dans la direction de la souris
</commit_message>
<xml_diff>
--- a/doc/JDT-P_OO.xlsx
+++ b/doc/JDT-P_OO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pi46vew\Documents\GitHub\P_OO-ShootMeUp-\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36EB7A0E-A7FB-44E6-9374-C70E22551C5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A9B7703-FC36-4FEA-B1AD-53130A1BDD73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="45">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -411,7 +411,7 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -467,10 +467,6 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -529,6 +525,32 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -573,32 +595,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -933,10 +929,10 @@
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="40" t="s">
+      <c r="B1" s="46" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="40"/>
+      <c r="C1" s="46"/>
       <c r="D1" s="8" t="s">
         <v>2</v>
       </c>
@@ -948,10 +944,10 @@
       <c r="A2" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="40" t="s">
+      <c r="B2" s="46" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="40"/>
+      <c r="C2" s="46"/>
       <c r="D2" s="8" t="s">
         <v>4</v>
       </c>
@@ -963,10 +959,10 @@
       <c r="A3" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="46" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="40"/>
+      <c r="C3" s="46"/>
       <c r="D3" s="8" t="s">
         <v>7</v>
       </c>
@@ -978,12 +974,12 @@
       <c r="A4" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="41" t="s">
+      <c r="B4" s="47" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="42"/>
-      <c r="D4" s="42"/>
-      <c r="E4" s="43"/>
+      <c r="C4" s="48"/>
+      <c r="D4" s="48"/>
+      <c r="E4" s="49"/>
     </row>
     <row r="5" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="16" t="s">
@@ -1006,16 +1002,16 @@
       <c r="A6" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="33">
+      <c r="B6" s="39">
         <v>45894</v>
       </c>
-      <c r="C6" s="20">
+      <c r="C6" s="19">
         <v>90</v>
       </c>
-      <c r="D6" s="22" t="s">
+      <c r="D6" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="E6" s="25" t="s">
+      <c r="E6" s="24" t="s">
         <v>30</v>
       </c>
     </row>
@@ -1023,14 +1019,14 @@
       <c r="A7" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="44"/>
+      <c r="B7" s="50"/>
       <c r="C7" s="9">
         <v>45</v>
       </c>
-      <c r="D7" s="23" t="s">
+      <c r="D7" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="E7" s="26" t="s">
+      <c r="E7" s="25" t="s">
         <v>30</v>
       </c>
     </row>
@@ -1038,14 +1034,14 @@
       <c r="A8" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="45"/>
-      <c r="C8" s="19">
+      <c r="B8" s="51"/>
+      <c r="C8" s="18">
         <v>45</v>
       </c>
-      <c r="D8" s="24" t="s">
+      <c r="D8" s="23" t="s">
         <v>24</v>
       </c>
-      <c r="E8" s="27" t="s">
+      <c r="E8" s="26" t="s">
         <v>30</v>
       </c>
     </row>
@@ -1053,28 +1049,28 @@
       <c r="A9" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="21"/>
-      <c r="C9" s="28">
+      <c r="B9" s="20"/>
+      <c r="C9" s="27">
         <f>SUM(C6:C8)</f>
         <v>180</v>
       </c>
-      <c r="D9" s="21"/>
-      <c r="E9" s="21"/>
+      <c r="D9" s="20"/>
+      <c r="E9" s="20"/>
     </row>
     <row r="10" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="B10" s="37">
+      <c r="B10" s="43">
         <v>46269</v>
       </c>
-      <c r="C10" s="20">
+      <c r="C10" s="19">
         <v>45</v>
       </c>
-      <c r="D10" s="17" t="s">
+      <c r="D10" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="E10" s="18" t="s">
+      <c r="E10" s="17" t="s">
         <v>30</v>
       </c>
     </row>
@@ -1082,14 +1078,14 @@
       <c r="A11" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="38"/>
+      <c r="B11" s="44"/>
       <c r="C11" s="9">
         <v>120</v>
       </c>
-      <c r="D11" s="17" t="s">
+      <c r="D11" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="E11" s="18" t="s">
+      <c r="E11" s="17" t="s">
         <v>32</v>
       </c>
     </row>
@@ -1097,14 +1093,14 @@
       <c r="A12" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="B12" s="39"/>
-      <c r="C12" s="19">
+      <c r="B12" s="45"/>
+      <c r="C12" s="18">
         <v>15</v>
       </c>
-      <c r="D12" s="17" t="s">
+      <c r="D12" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="E12" s="18" t="s">
+      <c r="E12" s="17" t="s">
         <v>30</v>
       </c>
     </row>
@@ -1112,149 +1108,186 @@
       <c r="A13" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="21"/>
-      <c r="C13" s="28">
+      <c r="B13" s="20"/>
+      <c r="C13" s="27">
         <f>SUM(C10:C12)</f>
         <v>180</v>
       </c>
-      <c r="D13" s="21"/>
-      <c r="E13" s="21"/>
+      <c r="D13" s="20"/>
+      <c r="E13" s="20"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="B14" s="33">
+      <c r="B14" s="39">
         <v>46276</v>
       </c>
-      <c r="C14" s="20">
+      <c r="C14" s="19">
         <v>60</v>
       </c>
-      <c r="D14" s="30" t="s">
+      <c r="D14" s="29" t="s">
         <v>34</v>
       </c>
-      <c r="E14" s="25" t="s">
+      <c r="E14" s="24" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="29" t="s">
+      <c r="A15" s="28" t="s">
         <v>37</v>
       </c>
-      <c r="B15" s="34"/>
-      <c r="C15" s="32">
+      <c r="B15" s="40"/>
+      <c r="C15" s="31">
         <v>20</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E15" s="26"/>
+      <c r="E15" s="25"/>
     </row>
     <row r="16" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="B16" s="34"/>
+      <c r="B16" s="40"/>
       <c r="C16" s="9">
         <v>10</v>
       </c>
-      <c r="D16" s="31" t="s">
+      <c r="D16" s="30" t="s">
         <v>36</v>
       </c>
-      <c r="E16" s="26"/>
+      <c r="E16" s="25"/>
     </row>
     <row r="17" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="52"/>
-      <c r="C17" s="28">
+      <c r="B17" s="38"/>
+      <c r="C17" s="27">
         <f>SUM(C14:C16)</f>
         <v>90</v>
       </c>
-      <c r="D17" s="21"/>
-      <c r="E17" s="21"/>
+      <c r="D17" s="20"/>
+      <c r="E17" s="20"/>
     </row>
     <row r="18" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="46" t="s">
+      <c r="A18" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="B18" s="33">
+      <c r="B18" s="39">
         <v>46283</v>
       </c>
-      <c r="C18" s="48">
+      <c r="C18" s="34">
         <v>50</v>
       </c>
-      <c r="D18" s="22" t="s">
+      <c r="D18" s="21" t="s">
         <v>41</v>
       </c>
-      <c r="E18" s="25"/>
+      <c r="E18" s="24"/>
     </row>
     <row r="19" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="29" t="s">
+      <c r="A19" s="28" t="s">
         <v>40</v>
       </c>
-      <c r="B19" s="34"/>
-      <c r="C19" s="49">
+      <c r="B19" s="40"/>
+      <c r="C19" s="35">
         <v>40</v>
       </c>
-      <c r="D19" s="51" t="s">
+      <c r="D19" s="37" t="s">
         <v>42</v>
       </c>
-      <c r="E19" s="26"/>
+      <c r="E19" s="25"/>
     </row>
     <row r="20" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="47" t="s">
+      <c r="A20" s="33" t="s">
         <v>40</v>
       </c>
-      <c r="B20" s="34"/>
-      <c r="C20" s="50">
+      <c r="B20" s="40"/>
+      <c r="C20" s="36">
         <v>30</v>
       </c>
-      <c r="D20" s="23" t="s">
+      <c r="D20" s="22" t="s">
         <v>43</v>
       </c>
-      <c r="E20" s="26"/>
+      <c r="E20" s="25"/>
     </row>
     <row r="21" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="47" t="s">
+      <c r="A21" s="33" t="s">
         <v>40</v>
       </c>
-      <c r="B21" s="34"/>
-      <c r="C21" s="49">
+      <c r="B21" s="40"/>
+      <c r="C21" s="35">
         <v>60</v>
       </c>
-      <c r="D21" s="51" t="s">
+      <c r="D21" s="37" t="s">
         <v>44</v>
       </c>
-      <c r="E21" s="51"/>
+      <c r="E21" s="37"/>
     </row>
     <row r="22" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B22" s="21"/>
-      <c r="C22" s="28">
+      <c r="B22" s="20"/>
+      <c r="C22" s="27">
         <f>SUM(C18:C21)</f>
         <v>180</v>
       </c>
-      <c r="D22" s="21"/>
-      <c r="E22" s="21"/>
-    </row>
-    <row r="23" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="24" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="25" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="26" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="27" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="D22" s="20"/>
+      <c r="E22" s="20"/>
+    </row>
+    <row r="23" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="32"/>
+      <c r="B23" s="39">
+        <v>46290</v>
+      </c>
+      <c r="C23" s="34"/>
+      <c r="D23" s="21"/>
+      <c r="E23" s="24"/>
+    </row>
+    <row r="24" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="28"/>
+      <c r="B24" s="40"/>
+      <c r="C24" s="35"/>
+      <c r="D24" s="37"/>
+      <c r="E24" s="25"/>
+    </row>
+    <row r="25" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="33"/>
+      <c r="B25" s="40"/>
+      <c r="C25" s="36"/>
+      <c r="D25" s="22"/>
+      <c r="E25" s="25"/>
+    </row>
+    <row r="26" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="33"/>
+      <c r="B26" s="40"/>
+      <c r="C26" s="35"/>
+      <c r="D26" s="37"/>
+      <c r="E26" s="37"/>
+    </row>
+    <row r="27" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B27" s="20"/>
+      <c r="C27" s="27">
+        <f>SUM(C23:C26)</f>
+        <v>0</v>
+      </c>
+      <c r="D27" s="20"/>
+      <c r="E27" s="20"/>
+    </row>
     <row r="28" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="29" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="30" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="31" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="32" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="35" t="s">
+      <c r="A32" s="41" t="s">
         <v>16</v>
       </c>
-      <c r="B32" s="36"/>
+      <c r="B32" s="42"/>
       <c r="C32" s="2">
         <f>MROUND(SUM(C6:C31) /60,0.2)</f>
         <v>21</v>
@@ -1281,7 +1314,7 @@
     <row r="49" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="50" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="10">
     <mergeCell ref="B14:B16"/>
     <mergeCell ref="A32:B32"/>
     <mergeCell ref="B10:B12"/>
@@ -1291,9 +1324,10 @@
     <mergeCell ref="B4:E4"/>
     <mergeCell ref="B6:B8"/>
     <mergeCell ref="B18:B21"/>
+    <mergeCell ref="B23:B26"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B6 C6:C8 B10 C10:C12 C16 B14:C14 C20 B18:C18" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B6 C6:C8 B10 C10:C12 C16 B14:C14 C20 B18:C18 C25 B23:C23" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -1330,6 +1364,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010051C931FEC57CD24D841BB655C8BA0DFF" ma:contentTypeVersion="14" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="f47e485f4ad8d247f3dfedaee1362e95">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3eb094ff-ec8d-44d8-be06-94ad3ec8832a" xmlns:ns3="4356f79f-5386-4bda-9d92-82d8bd7b074e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="da34bf24383b1ce13aa9c82f6b8627bb" ns2:_="" ns3:_="">
     <xsd:import namespace="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
@@ -1542,15 +1585,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
   <ds:schemaRefs>
@@ -1569,6 +1603,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5A40649F-4D7C-4B62-9A51-E0A7D9450EFE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1585,12 +1627,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
refactor(attaque burger) relocalisation de la logique de tir
</commit_message>
<xml_diff>
--- a/doc/JDT-P_OO.xlsx
+++ b/doc/JDT-P_OO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pi46vew\Documents\GitHub\P_OO-ShootMeUp-\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A9B7703-FC36-4FEA-B1AD-53130A1BDD73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DC6F604-9DAC-4E73-A767-E7331AF05706}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="48">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -185,6 +185,15 @@
   </si>
   <si>
     <t>Instantiation du burger sur la carte lors du clique mais pas réussi à ajouter la trajectoire (User Story num 2)</t>
+  </si>
+  <si>
+    <t>Les attauques burger vont en direction de la souris</t>
+  </si>
+  <si>
+    <t>Ajout d'un cooldown aux tirs burger</t>
+  </si>
+  <si>
+    <t>les burgers sont detruit si ils touches les bords du gamespace</t>
   </si>
 </sst>
 </file>
@@ -1238,26 +1247,44 @@
       <c r="E22" s="20"/>
     </row>
     <row r="23" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="32"/>
+      <c r="A23" s="32" t="s">
+        <v>40</v>
+      </c>
       <c r="B23" s="39">
         <v>46290</v>
       </c>
-      <c r="C23" s="34"/>
-      <c r="D23" s="21"/>
+      <c r="C23" s="34">
+        <v>45</v>
+      </c>
+      <c r="D23" s="21" t="s">
+        <v>45</v>
+      </c>
       <c r="E23" s="24"/>
     </row>
     <row r="24" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="28"/>
+      <c r="A24" s="28" t="s">
+        <v>40</v>
+      </c>
       <c r="B24" s="40"/>
-      <c r="C24" s="35"/>
-      <c r="D24" s="37"/>
+      <c r="C24" s="35">
+        <v>20</v>
+      </c>
+      <c r="D24" s="37" t="s">
+        <v>46</v>
+      </c>
       <c r="E24" s="25"/>
     </row>
     <row r="25" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="33"/>
+      <c r="A25" s="33" t="s">
+        <v>40</v>
+      </c>
       <c r="B25" s="40"/>
-      <c r="C25" s="36"/>
-      <c r="D25" s="22"/>
+      <c r="C25" s="36">
+        <v>25</v>
+      </c>
+      <c r="D25" s="22" t="s">
+        <v>47</v>
+      </c>
       <c r="E25" s="25"/>
     </row>
     <row r="26" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1274,7 +1301,7 @@
       <c r="B27" s="20"/>
       <c r="C27" s="27">
         <f>SUM(C23:C26)</f>
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="D27" s="20"/>
       <c r="E27" s="20"/>
@@ -1290,7 +1317,7 @@
       <c r="B32" s="42"/>
       <c r="C32" s="2">
         <f>MROUND(SUM(C6:C31) /60,0.2)</f>
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D32" s="3"/>
       <c r="E32" s="4"/>

</xml_diff>

<commit_message>
feat(attque melee) ajout de couleur pour montrer l'attaque
</commit_message>
<xml_diff>
--- a/doc/JDT-P_OO.xlsx
+++ b/doc/JDT-P_OO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pi46vew\Documents\GitHub\P_OO-ShootMeUp-\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DC6F604-9DAC-4E73-A767-E7331AF05706}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADC62512-087F-43E5-8EF6-36CF45D963BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="50">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -194,6 +194,12 @@
   </si>
   <si>
     <t>les burgers sont detruit si ils touches les bords du gamespace</t>
+  </si>
+  <si>
+    <t>Attaque mélée</t>
+  </si>
+  <si>
+    <t>Ajout d'une attaque d'un mode "mélée" pour le joueur quand il fait une attaque mélée</t>
   </si>
 </sst>
 </file>
@@ -420,7 +426,7 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -603,6 +609,13 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
@@ -1253,7 +1266,7 @@
       <c r="B23" s="39">
         <v>46290</v>
       </c>
-      <c r="C23" s="34">
+      <c r="C23" s="19">
         <v>45</v>
       </c>
       <c r="D23" s="21" t="s">
@@ -1266,7 +1279,7 @@
         <v>40</v>
       </c>
       <c r="B24" s="40"/>
-      <c r="C24" s="35">
+      <c r="C24" s="31">
         <v>20</v>
       </c>
       <c r="D24" s="37" t="s">
@@ -1279,7 +1292,7 @@
         <v>40</v>
       </c>
       <c r="B25" s="40"/>
-      <c r="C25" s="36">
+      <c r="C25" s="9">
         <v>25</v>
       </c>
       <c r="D25" s="22" t="s">
@@ -1287,26 +1300,37 @@
       </c>
       <c r="E25" s="25"/>
     </row>
-    <row r="26" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="33"/>
+    <row r="26" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="33" t="s">
+        <v>48</v>
+      </c>
       <c r="B26" s="40"/>
-      <c r="C26" s="35"/>
-      <c r="D26" s="37"/>
+      <c r="C26" s="31">
+        <v>45</v>
+      </c>
+      <c r="D26" s="37" t="s">
+        <v>49</v>
+      </c>
       <c r="E26" s="37"/>
     </row>
     <row r="27" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="10" t="s">
+      <c r="B27" s="53"/>
+      <c r="C27" s="52"/>
+      <c r="D27" s="52"/>
+      <c r="E27" s="52"/>
+    </row>
+    <row r="28" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B27" s="20"/>
-      <c r="C27" s="27">
-        <f>SUM(C23:C26)</f>
-        <v>90</v>
-      </c>
-      <c r="D27" s="20"/>
-      <c r="E27" s="20"/>
-    </row>
-    <row r="28" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="B28" s="20"/>
+      <c r="C28" s="27">
+        <f>SUM(C23:C27)</f>
+        <v>135</v>
+      </c>
+      <c r="D28" s="20"/>
+      <c r="E28" s="20"/>
+    </row>
     <row r="29" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="30" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="31" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
@@ -1317,7 +1341,7 @@
       <c r="B32" s="42"/>
       <c r="C32" s="2">
         <f>MROUND(SUM(C6:C31) /60,0.2)</f>
-        <v>24</v>
+        <v>25.6</v>
       </c>
       <c r="D32" s="3"/>
       <c r="E32" s="4"/>
@@ -1351,9 +1375,9 @@
     <mergeCell ref="B4:E4"/>
     <mergeCell ref="B6:B8"/>
     <mergeCell ref="B18:B21"/>
-    <mergeCell ref="B23:B26"/>
+    <mergeCell ref="B23:B27"/>
   </mergeCells>
-  <dataValidations count="1">
+  <dataValidations disablePrompts="1" count="1">
     <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B6 C6:C8 B10 C10:C12 C16 B14:C14 C20 B18:C18 C25 B23:C23" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
       <formula1>0</formula1>
     </dataValidation>

</xml_diff>

<commit_message>
chore(JDT) mise à jour du journal de travail
</commit_message>
<xml_diff>
--- a/doc/JDT-P_OO.xlsx
+++ b/doc/JDT-P_OO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pi46vew\Documents\GitHub\P_OO-ShootMeUp-\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADC62512-087F-43E5-8EF6-36CF45D963BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B16E94F-2384-4E34-B949-8739702E1C8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$32</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$37</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="52">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -200,6 +200,12 @@
   </si>
   <si>
     <t>Ajout d'une attaque d'un mode "mélée" pour le joueur quand il fait une attaque mélée</t>
+  </si>
+  <si>
+    <t>Manager</t>
+  </si>
+  <si>
+    <t>Commencer l'ajout d'un enemie de type Manager. Création de la classe et des premiers attributs</t>
   </si>
 </sst>
 </file>
@@ -426,7 +432,7 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -613,11 +619,14 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1306,7 +1315,7 @@
       </c>
       <c r="B26" s="40"/>
       <c r="C26" s="31">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="D26" s="37" t="s">
         <v>49</v>
@@ -1314,9 +1323,16 @@
       <c r="E26" s="37"/>
     </row>
     <row r="27" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="28" t="s">
+        <v>50</v>
+      </c>
       <c r="B27" s="53"/>
-      <c r="C27" s="52"/>
-      <c r="D27" s="52"/>
+      <c r="C27" s="52">
+        <v>30</v>
+      </c>
+      <c r="D27" s="54" t="s">
+        <v>51</v>
+      </c>
       <c r="E27" s="52"/>
     </row>
     <row r="28" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1326,26 +1342,26 @@
       <c r="B28" s="20"/>
       <c r="C28" s="27">
         <f>SUM(C23:C27)</f>
-        <v>135</v>
+        <v>180</v>
       </c>
       <c r="D28" s="20"/>
       <c r="E28" s="20"/>
     </row>
-    <row r="29" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="29" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="41" t="s">
+        <v>16</v>
+      </c>
+      <c r="B29" s="42"/>
+      <c r="C29" s="2">
+        <f>MROUND(SUM(C9,C13,C17,C22,C28) /60,0.2)</f>
+        <v>13.600000000000001</v>
+      </c>
+      <c r="D29" s="3"/>
+      <c r="E29" s="4"/>
+    </row>
     <row r="30" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="31" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="32" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="41" t="s">
-        <v>16</v>
-      </c>
-      <c r="B32" s="42"/>
-      <c r="C32" s="2">
-        <f>MROUND(SUM(C6:C31) /60,0.2)</f>
-        <v>25.6</v>
-      </c>
-      <c r="D32" s="3"/>
-      <c r="E32" s="4"/>
-    </row>
+    <row r="31" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="32" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="33" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="34" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="35" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -1367,7 +1383,7 @@
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="B14:B16"/>
-    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="A29:B29"/>
     <mergeCell ref="B10:B12"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>

</xml_diff>

<commit_message>
feat(manager) ajout d'un système de dégat avec PV et dégat reçu des armes
</commit_message>
<xml_diff>
--- a/doc/JDT-P_OO.xlsx
+++ b/doc/JDT-P_OO.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30430"/>
   <workbookPr updateLinks="never" codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pi46vew\Documents\GitHub\P_OO-ShootMeUp-\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B16E94F-2384-4E34-B949-8739702E1C8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0901A7AB-3105-48C8-B92E-D1863D5B077B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="54">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -206,6 +206,12 @@
   </si>
   <si>
     <t>Commencer l'ajout d'un enemie de type Manager. Création de la classe et des premiers attributs</t>
+  </si>
+  <si>
+    <t>Ajout d'un déplacement aléatoire des managers</t>
+  </si>
+  <si>
+    <t>Ajout d'une barre de vie au manager</t>
   </si>
 </sst>
 </file>
@@ -432,7 +438,7 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -572,6 +578,12 @@
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -618,15 +630,27 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -960,10 +984,10 @@
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="46" t="s">
+      <c r="B1" s="48" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="46"/>
+      <c r="C1" s="48"/>
       <c r="D1" s="8" t="s">
         <v>2</v>
       </c>
@@ -975,10 +999,10 @@
       <c r="A2" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="46" t="s">
+      <c r="B2" s="48" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="46"/>
+      <c r="C2" s="48"/>
       <c r="D2" s="8" t="s">
         <v>4</v>
       </c>
@@ -990,10 +1014,10 @@
       <c r="A3" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="46" t="s">
+      <c r="B3" s="48" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="46"/>
+      <c r="C3" s="48"/>
       <c r="D3" s="8" t="s">
         <v>7</v>
       </c>
@@ -1005,12 +1029,12 @@
       <c r="A4" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="47" t="s">
+      <c r="B4" s="49" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="48"/>
-      <c r="D4" s="48"/>
-      <c r="E4" s="49"/>
+      <c r="C4" s="50"/>
+      <c r="D4" s="50"/>
+      <c r="E4" s="51"/>
     </row>
     <row r="5" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="16" t="s">
@@ -1033,7 +1057,7 @@
       <c r="A6" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="39">
+      <c r="B6" s="41">
         <v>45894</v>
       </c>
       <c r="C6" s="19">
@@ -1050,7 +1074,7 @@
       <c r="A7" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="50"/>
+      <c r="B7" s="52"/>
       <c r="C7" s="9">
         <v>45</v>
       </c>
@@ -1065,7 +1089,7 @@
       <c r="A8" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="51"/>
+      <c r="B8" s="53"/>
       <c r="C8" s="18">
         <v>45</v>
       </c>
@@ -1092,7 +1116,7 @@
       <c r="A10" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="B10" s="43">
+      <c r="B10" s="45">
         <v>46269</v>
       </c>
       <c r="C10" s="19">
@@ -1109,7 +1133,7 @@
       <c r="A11" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="44"/>
+      <c r="B11" s="46"/>
       <c r="C11" s="9">
         <v>120</v>
       </c>
@@ -1124,7 +1148,7 @@
       <c r="A12" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="B12" s="45"/>
+      <c r="B12" s="47"/>
       <c r="C12" s="18">
         <v>15</v>
       </c>
@@ -1151,7 +1175,7 @@
       <c r="A14" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="B14" s="39">
+      <c r="B14" s="41">
         <v>46276</v>
       </c>
       <c r="C14" s="19">
@@ -1168,7 +1192,7 @@
       <c r="A15" s="28" t="s">
         <v>37</v>
       </c>
-      <c r="B15" s="40"/>
+      <c r="B15" s="42"/>
       <c r="C15" s="31">
         <v>20</v>
       </c>
@@ -1181,7 +1205,7 @@
       <c r="A16" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="B16" s="40"/>
+      <c r="B16" s="42"/>
       <c r="C16" s="9">
         <v>10</v>
       </c>
@@ -1206,7 +1230,7 @@
       <c r="A18" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="B18" s="39">
+      <c r="B18" s="41">
         <v>46283</v>
       </c>
       <c r="C18" s="34">
@@ -1221,7 +1245,7 @@
       <c r="A19" s="28" t="s">
         <v>40</v>
       </c>
-      <c r="B19" s="40"/>
+      <c r="B19" s="42"/>
       <c r="C19" s="35">
         <v>40</v>
       </c>
@@ -1234,7 +1258,7 @@
       <c r="A20" s="33" t="s">
         <v>40</v>
       </c>
-      <c r="B20" s="40"/>
+      <c r="B20" s="42"/>
       <c r="C20" s="36">
         <v>30</v>
       </c>
@@ -1247,7 +1271,7 @@
       <c r="A21" s="33" t="s">
         <v>40</v>
       </c>
-      <c r="B21" s="40"/>
+      <c r="B21" s="42"/>
       <c r="C21" s="35">
         <v>60</v>
       </c>
@@ -1272,7 +1296,7 @@
       <c r="A23" s="32" t="s">
         <v>40</v>
       </c>
-      <c r="B23" s="39">
+      <c r="B23" s="41">
         <v>46290</v>
       </c>
       <c r="C23" s="19">
@@ -1287,7 +1311,7 @@
       <c r="A24" s="28" t="s">
         <v>40</v>
       </c>
-      <c r="B24" s="40"/>
+      <c r="B24" s="42"/>
       <c r="C24" s="31">
         <v>20</v>
       </c>
@@ -1300,7 +1324,7 @@
       <c r="A25" s="33" t="s">
         <v>40</v>
       </c>
-      <c r="B25" s="40"/>
+      <c r="B25" s="42"/>
       <c r="C25" s="9">
         <v>25</v>
       </c>
@@ -1313,7 +1337,7 @@
       <c r="A26" s="33" t="s">
         <v>48</v>
       </c>
-      <c r="B26" s="40"/>
+      <c r="B26" s="42"/>
       <c r="C26" s="31">
         <v>60</v>
       </c>
@@ -1326,14 +1350,14 @@
       <c r="A27" s="28" t="s">
         <v>50</v>
       </c>
-      <c r="B27" s="53"/>
-      <c r="C27" s="52">
+      <c r="B27" s="54"/>
+      <c r="C27" s="39">
         <v>30</v>
       </c>
-      <c r="D27" s="54" t="s">
+      <c r="D27" s="40" t="s">
         <v>51</v>
       </c>
-      <c r="E27" s="52"/>
+      <c r="E27" s="39"/>
     </row>
     <row r="28" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="10" t="s">
@@ -1347,43 +1371,98 @@
       <c r="D28" s="20"/>
       <c r="E28" s="20"/>
     </row>
-    <row r="29" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="41" t="s">
+    <row r="29" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="57" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29" s="60">
+        <v>46297</v>
+      </c>
+      <c r="C29" s="57">
+        <v>45</v>
+      </c>
+      <c r="D29" s="55" t="s">
+        <v>52</v>
+      </c>
+      <c r="E29" s="55"/>
+    </row>
+    <row r="30" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="31" t="s">
+        <v>50</v>
+      </c>
+      <c r="B30" s="58"/>
+      <c r="C30" s="31">
+        <v>45</v>
+      </c>
+      <c r="D30" s="37" t="s">
+        <v>53</v>
+      </c>
+      <c r="E30" s="37"/>
+    </row>
+    <row r="31" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="31"/>
+      <c r="B31" s="58"/>
+      <c r="C31" s="31"/>
+      <c r="D31" s="37"/>
+      <c r="E31" s="37"/>
+    </row>
+    <row r="32" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="31"/>
+      <c r="B32" s="58"/>
+      <c r="C32" s="31"/>
+      <c r="D32" s="37"/>
+      <c r="E32" s="37"/>
+    </row>
+    <row r="33" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="39"/>
+      <c r="B33" s="59"/>
+      <c r="C33" s="39"/>
+      <c r="D33" s="56"/>
+      <c r="E33" s="56"/>
+    </row>
+    <row r="34" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B34" s="20"/>
+      <c r="C34" s="27">
+        <f>SUM(C29:C33)</f>
+        <v>90</v>
+      </c>
+      <c r="D34" s="20"/>
+      <c r="E34" s="20"/>
+    </row>
+    <row r="35" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="B29" s="42"/>
-      <c r="C29" s="2">
+      <c r="B35" s="44"/>
+      <c r="C35" s="2">
         <f>MROUND(SUM(C9,C13,C17,C22,C28) /60,0.2)</f>
         <v>13.600000000000001</v>
       </c>
-      <c r="D29" s="3"/>
-      <c r="E29" s="4"/>
-    </row>
-    <row r="30" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="31" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="32" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="33" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="34" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="35" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="36" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="37" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="38" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="39" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="40" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="43" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="44" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="45" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="46" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="47" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="48" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="D35" s="3"/>
+      <c r="E35" s="4"/>
+    </row>
+    <row r="36" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="37" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="38" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="39" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="40" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="41" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="42" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="43" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="44" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="45" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="46" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="47" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="48" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="49" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="50" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
     <mergeCell ref="B14:B16"/>
-    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A35:B35"/>
     <mergeCell ref="B10:B12"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
@@ -1392,6 +1471,7 @@
     <mergeCell ref="B6:B8"/>
     <mergeCell ref="B18:B21"/>
     <mergeCell ref="B23:B27"/>
+    <mergeCell ref="B29:B33"/>
   </mergeCells>
   <dataValidations disablePrompts="1" count="1">
     <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B6 C6:C8 B10 C10:C12 C16 B14:C14 C20 B18:C18 C25 B23:C23" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
@@ -1431,15 +1511,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010051C931FEC57CD24D841BB655C8BA0DFF" ma:contentTypeVersion="14" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="f47e485f4ad8d247f3dfedaee1362e95">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3eb094ff-ec8d-44d8-be06-94ad3ec8832a" xmlns:ns3="4356f79f-5386-4bda-9d92-82d8bd7b074e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="da34bf24383b1ce13aa9c82f6b8627bb" ns2:_="" ns3:_="">
     <xsd:import namespace="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
@@ -1652,6 +1723,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
   <ds:schemaRefs>
@@ -1670,14 +1750,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5A40649F-4D7C-4B62-9A51-E0A7D9450EFE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1694,4 +1766,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
chore(JDT) mise a jour du journal de travail
</commit_message>
<xml_diff>
--- a/doc/JDT-P_OO.xlsx
+++ b/doc/JDT-P_OO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pi46vew\Documents\GitHub\P_OO-ShootMeUp-\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0901A7AB-3105-48C8-B92E-D1863D5B077B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9CDD9AC-B1CA-4859-95C8-568236926AED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="58">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -212,6 +212,18 @@
   </si>
   <si>
     <t>Ajout d'une barre de vie au manager</t>
+  </si>
+  <si>
+    <t>barre de vie</t>
+  </si>
+  <si>
+    <t>Création d'une barre de vie et d un écran de mort quand les PV passe à 0</t>
+  </si>
+  <si>
+    <t>barre d'argent</t>
+  </si>
+  <si>
+    <t>Commencer la création d'une barre d'argent pour pouvoir gagner</t>
   </si>
 </sst>
 </file>
@@ -1400,21 +1412,32 @@
       <c r="E30" s="37"/>
     </row>
     <row r="31" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="31"/>
+      <c r="A31" s="31" t="s">
+        <v>54</v>
+      </c>
       <c r="B31" s="58"/>
-      <c r="C31" s="31"/>
-      <c r="D31" s="37"/>
+      <c r="C31" s="31">
+        <v>60</v>
+      </c>
+      <c r="D31" s="37" t="s">
+        <v>55</v>
+      </c>
       <c r="E31" s="37"/>
     </row>
     <row r="32" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="31"/>
+      <c r="A32" s="31" t="s">
+        <v>56</v>
+      </c>
       <c r="B32" s="58"/>
-      <c r="C32" s="31"/>
-      <c r="D32" s="37"/>
+      <c r="C32" s="31">
+        <v>30</v>
+      </c>
+      <c r="D32" s="37" t="s">
+        <v>57</v>
+      </c>
       <c r="E32" s="37"/>
     </row>
     <row r="33" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="39"/>
       <c r="B33" s="59"/>
       <c r="C33" s="39"/>
       <c r="D33" s="56"/>
@@ -1427,7 +1450,7 @@
       <c r="B34" s="20"/>
       <c r="C34" s="27">
         <f>SUM(C29:C33)</f>
-        <v>90</v>
+        <v>180</v>
       </c>
       <c r="D34" s="20"/>
       <c r="E34" s="20"/>

</xml_diff>

<commit_message>
WIP(obstacle) créée les obstacle mais pas encore de détection de collision
</commit_message>
<xml_diff>
--- a/doc/JDT-P_OO.xlsx
+++ b/doc/JDT-P_OO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pi46vew\Documents\GitHub\P_OO-ShootMeUp-\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74B2F06F-88A4-46FA-91A5-EE9054E7D5E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E87B0038-0B8A-453A-8D58-7CD2028DBC27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$43</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$39</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="64">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -230,6 +230,18 @@
   </si>
   <si>
     <t>Création d'un ennemi robot en s'inspirant beacoup de l'ennemi manager</t>
+  </si>
+  <si>
+    <t>Faisceau</t>
+  </si>
+  <si>
+    <t>Création d'un faisceau pouvant aller dans les quatres direction</t>
+  </si>
+  <si>
+    <t>Fait en sorte que les faisceaux fassent des dégats quand ils touches le joueur et qu'ils soit tirés par les robots</t>
+  </si>
+  <si>
+    <t>Commencer la création des obstacles</t>
   </si>
 </sst>
 </file>
@@ -992,7 +1004,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33" style="1" customWidth="1"/>
@@ -1469,7 +1481,7 @@
         <v>46304</v>
       </c>
       <c r="C34" s="43">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="D34" s="41" t="s">
         <v>59</v>
@@ -1477,24 +1489,38 @@
       <c r="E34" s="41"/>
     </row>
     <row r="35" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="31"/>
+      <c r="A35" s="31" t="s">
+        <v>60</v>
+      </c>
       <c r="B35" s="59"/>
-      <c r="C35" s="31"/>
-      <c r="D35" s="37"/>
+      <c r="C35" s="31">
+        <v>50</v>
+      </c>
+      <c r="D35" s="37" t="s">
+        <v>61</v>
+      </c>
       <c r="E35" s="37"/>
     </row>
     <row r="36" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="31"/>
       <c r="B36" s="59"/>
-      <c r="C36" s="31"/>
-      <c r="D36" s="37"/>
+      <c r="C36" s="31">
+        <v>45</v>
+      </c>
+      <c r="D36" s="37" t="s">
+        <v>62</v>
+      </c>
       <c r="E36" s="37"/>
     </row>
     <row r="37" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="39"/>
       <c r="B37" s="60"/>
-      <c r="C37" s="39"/>
-      <c r="D37" s="42"/>
+      <c r="C37" s="39">
+        <v>25</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>63</v>
+      </c>
       <c r="E37" s="42"/>
     </row>
     <row r="38" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1504,38 +1530,35 @@
       <c r="B38" s="20"/>
       <c r="C38" s="27">
         <f>SUM(C34:C37)</f>
-        <v>45</v>
+        <v>180</v>
       </c>
       <c r="D38" s="20"/>
       <c r="E38" s="20"/>
     </row>
-    <row r="39" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="39" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="46" t="s">
+        <v>16</v>
+      </c>
+      <c r="B39" s="47"/>
+      <c r="C39" s="2">
+        <f>MROUND(SUM(C9,C13,C17,C22,C28,C33,C38) /60,0.2)</f>
+        <v>19.600000000000001</v>
+      </c>
+      <c r="D39" s="3"/>
+      <c r="E39" s="4"/>
+    </row>
     <row r="40" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="41" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="43" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="46" t="s">
-        <v>16</v>
-      </c>
-      <c r="B43" s="47"/>
-      <c r="C43" s="2">
-        <f>MROUND(SUM(C9,C13,C17,C22,C28) /60,0.2)</f>
-        <v>13.600000000000001</v>
-      </c>
-      <c r="D43" s="3"/>
-      <c r="E43" s="4"/>
-    </row>
+    <row r="42" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="43" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="44" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="45" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="46" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="47" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="48" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="49" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="50" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="47" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="12">
     <mergeCell ref="B14:B16"/>
-    <mergeCell ref="A43:B43"/>
+    <mergeCell ref="A39:B39"/>
     <mergeCell ref="B10:B12"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>

</xml_diff>

<commit_message>
doc(rapport) avancé dans le diagramme de classe
</commit_message>
<xml_diff>
--- a/doc/JDT-P_OO.xlsx
+++ b/doc/JDT-P_OO.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30527"/>
   <workbookPr updateLinks="never" codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pi46vew\Documents\GitHub\P_OO-ShootMeUp-\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{136A932E-0372-412C-9314-14F00B6816A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{602A9E34-BAA7-4B82-97A0-94B5873DE484}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$39</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$58</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="71">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -245,6 +245,24 @@
   </si>
   <si>
     <t>Obstacle</t>
+  </si>
+  <si>
+    <t>Finis la création des obstacles et fait en sorte que les Manager et Robot trouve un nouveau chemin</t>
+  </si>
+  <si>
+    <t>Tests</t>
+  </si>
+  <si>
+    <t>Ecriture des HelpersTests</t>
+  </si>
+  <si>
+    <t>Ecriture de PlayerTests</t>
+  </si>
+  <si>
+    <t>Ecriture de ManagerTests</t>
+  </si>
+  <si>
+    <t>Ecriture de RobotTests</t>
   </si>
 </sst>
 </file>
@@ -482,7 +500,7 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -619,6 +637,15 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -626,6 +653,9 @@
     <xf numFmtId="14" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
@@ -681,17 +711,22 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1009,7 +1044,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E58"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33" style="1" customWidth="1"/>
@@ -1025,10 +1060,10 @@
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="45" t="s">
+      <c r="B1" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="45"/>
+      <c r="C1" s="49"/>
       <c r="D1" s="8" t="s">
         <v>2</v>
       </c>
@@ -1040,10 +1075,10 @@
       <c r="A2" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="45" t="s">
+      <c r="B2" s="49" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="45"/>
+      <c r="C2" s="49"/>
       <c r="D2" s="8" t="s">
         <v>4</v>
       </c>
@@ -1055,10 +1090,10 @@
       <c r="A3" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="45" t="s">
+      <c r="B3" s="49" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="45"/>
+      <c r="C3" s="49"/>
       <c r="D3" s="8" t="s">
         <v>7</v>
       </c>
@@ -1070,27 +1105,27 @@
       <c r="A4" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="46" t="s">
+      <c r="B4" s="50" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="47"/>
-      <c r="D4" s="47"/>
-      <c r="E4" s="48"/>
+      <c r="C4" s="51"/>
+      <c r="D4" s="51"/>
+      <c r="E4" s="52"/>
     </row>
     <row r="5" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="58" t="s">
+      <c r="A5" s="39" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="59" t="s">
+      <c r="B5" s="40" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="59" t="s">
+      <c r="C5" s="40" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="59" t="s">
+      <c r="D5" s="40" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="60" t="s">
+      <c r="E5" s="41" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1098,7 +1133,7 @@
       <c r="A6" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="39">
+      <c r="B6" s="42">
         <v>45894</v>
       </c>
       <c r="C6" s="17">
@@ -1115,7 +1150,7 @@
       <c r="A7" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="49"/>
+      <c r="B7" s="53"/>
       <c r="C7" s="9">
         <v>45</v>
       </c>
@@ -1130,7 +1165,7 @@
       <c r="A8" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="50"/>
+      <c r="B8" s="54"/>
       <c r="C8" s="16">
         <v>45</v>
       </c>
@@ -1157,7 +1192,7 @@
       <c r="A10" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="B10" s="42">
+      <c r="B10" s="46">
         <v>46269</v>
       </c>
       <c r="C10" s="17">
@@ -1174,7 +1209,7 @@
       <c r="A11" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="43"/>
+      <c r="B11" s="47"/>
       <c r="C11" s="9">
         <v>120</v>
       </c>
@@ -1189,7 +1224,7 @@
       <c r="A12" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="B12" s="44"/>
+      <c r="B12" s="48"/>
       <c r="C12" s="16">
         <v>15</v>
       </c>
@@ -1216,7 +1251,7 @@
       <c r="A14" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="B14" s="39">
+      <c r="B14" s="42">
         <v>46276</v>
       </c>
       <c r="C14" s="17">
@@ -1233,7 +1268,7 @@
       <c r="A15" s="28" t="s">
         <v>37</v>
       </c>
-      <c r="B15" s="40"/>
+      <c r="B15" s="43"/>
       <c r="C15" s="28">
         <v>20</v>
       </c>
@@ -1246,7 +1281,7 @@
       <c r="A16" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="B16" s="40"/>
+      <c r="B16" s="43"/>
       <c r="C16" s="9">
         <v>10</v>
       </c>
@@ -1271,7 +1306,7 @@
       <c r="A18" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="B18" s="39">
+      <c r="B18" s="42">
         <v>46283</v>
       </c>
       <c r="C18" s="29">
@@ -1286,7 +1321,7 @@
       <c r="A19" s="28" t="s">
         <v>40</v>
       </c>
-      <c r="B19" s="40"/>
+      <c r="B19" s="43"/>
       <c r="C19" s="30">
         <v>40</v>
       </c>
@@ -1299,7 +1334,7 @@
       <c r="A20" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="B20" s="40"/>
+      <c r="B20" s="43"/>
       <c r="C20" s="31">
         <v>30</v>
       </c>
@@ -1312,7 +1347,7 @@
       <c r="A21" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="B21" s="40"/>
+      <c r="B21" s="43"/>
       <c r="C21" s="30">
         <v>60</v>
       </c>
@@ -1337,7 +1372,7 @@
       <c r="A23" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="B23" s="39">
+      <c r="B23" s="42">
         <v>46290</v>
       </c>
       <c r="C23" s="17">
@@ -1352,7 +1387,7 @@
       <c r="A24" s="28" t="s">
         <v>40</v>
       </c>
-      <c r="B24" s="40"/>
+      <c r="B24" s="43"/>
       <c r="C24" s="28">
         <v>20</v>
       </c>
@@ -1365,7 +1400,7 @@
       <c r="A25" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="B25" s="40"/>
+      <c r="B25" s="43"/>
       <c r="C25" s="9">
         <v>25</v>
       </c>
@@ -1378,7 +1413,7 @@
       <c r="A26" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="B26" s="40"/>
+      <c r="B26" s="43"/>
       <c r="C26" s="28">
         <v>60</v>
       </c>
@@ -1391,7 +1426,7 @@
       <c r="A27" s="28" t="s">
         <v>50</v>
       </c>
-      <c r="B27" s="51"/>
+      <c r="B27" s="55"/>
       <c r="C27" s="34">
         <v>30</v>
       </c>
@@ -1416,7 +1451,7 @@
       <c r="A29" s="38" t="s">
         <v>50</v>
       </c>
-      <c r="B29" s="52">
+      <c r="B29" s="56">
         <v>46297</v>
       </c>
       <c r="C29" s="38">
@@ -1431,7 +1466,7 @@
       <c r="A30" s="28" t="s">
         <v>50</v>
       </c>
-      <c r="B30" s="53"/>
+      <c r="B30" s="57"/>
       <c r="C30" s="28">
         <v>45</v>
       </c>
@@ -1444,7 +1479,7 @@
       <c r="A31" s="28" t="s">
         <v>54</v>
       </c>
-      <c r="B31" s="53"/>
+      <c r="B31" s="57"/>
       <c r="C31" s="28">
         <v>60</v>
       </c>
@@ -1457,7 +1492,7 @@
       <c r="A32" s="28" t="s">
         <v>56</v>
       </c>
-      <c r="B32" s="54"/>
+      <c r="B32" s="58"/>
       <c r="C32" s="28">
         <v>30</v>
       </c>
@@ -1482,7 +1517,7 @@
       <c r="A34" s="38" t="s">
         <v>58</v>
       </c>
-      <c r="B34" s="52">
+      <c r="B34" s="56">
         <v>46304</v>
       </c>
       <c r="C34" s="38">
@@ -1497,7 +1532,7 @@
       <c r="A35" s="28" t="s">
         <v>60</v>
       </c>
-      <c r="B35" s="55"/>
+      <c r="B35" s="59"/>
       <c r="C35" s="28">
         <v>50</v>
       </c>
@@ -1510,7 +1545,7 @@
       <c r="A36" s="28" t="s">
         <v>60</v>
       </c>
-      <c r="B36" s="55"/>
+      <c r="B36" s="59"/>
       <c r="C36" s="28">
         <v>45</v>
       </c>
@@ -1523,7 +1558,7 @@
       <c r="A37" s="34" t="s">
         <v>64</v>
       </c>
-      <c r="B37" s="56"/>
+      <c r="B37" s="60"/>
       <c r="C37" s="34">
         <v>25</v>
       </c>
@@ -1544,30 +1579,151 @@
       <c r="D38" s="18"/>
       <c r="E38" s="18"/>
     </row>
-    <row r="39" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="57" t="s">
+    <row r="39" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="62" t="s">
+        <v>64</v>
+      </c>
+      <c r="B39" s="56">
+        <v>46318</v>
+      </c>
+      <c r="C39" s="38">
+        <v>60</v>
+      </c>
+      <c r="D39" s="36" t="s">
+        <v>65</v>
+      </c>
+      <c r="E39" s="36"/>
+    </row>
+    <row r="40" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="63" t="s">
+        <v>66</v>
+      </c>
+      <c r="B40" s="57"/>
+      <c r="C40" s="28">
+        <v>20</v>
+      </c>
+      <c r="D40" s="32" t="s">
+        <v>67</v>
+      </c>
+      <c r="E40" s="32"/>
+    </row>
+    <row r="41" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="63" t="s">
+        <v>66</v>
+      </c>
+      <c r="B41" s="57"/>
+      <c r="C41" s="28">
+        <v>40</v>
+      </c>
+      <c r="D41" s="32" t="s">
+        <v>68</v>
+      </c>
+      <c r="E41" s="32"/>
+    </row>
+    <row r="42" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="63" t="s">
+        <v>66</v>
+      </c>
+      <c r="B42" s="57"/>
+      <c r="C42" s="28">
+        <v>30</v>
+      </c>
+      <c r="D42" s="32" t="s">
+        <v>69</v>
+      </c>
+      <c r="E42" s="32"/>
+    </row>
+    <row r="43" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="61" t="s">
+        <v>66</v>
+      </c>
+      <c r="B43" s="58"/>
+      <c r="C43" s="34">
+        <v>30</v>
+      </c>
+      <c r="D43" s="37" t="s">
+        <v>70</v>
+      </c>
+      <c r="E43" s="37"/>
+    </row>
+    <row r="44" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B44" s="18"/>
+      <c r="C44" s="64">
+        <f>SUM(C39:C43)</f>
+        <v>180</v>
+      </c>
+      <c r="D44" s="65"/>
+      <c r="E44" s="65"/>
+    </row>
+    <row r="45" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="62"/>
+      <c r="B45" s="56">
+        <v>46325</v>
+      </c>
+      <c r="C45" s="38"/>
+      <c r="D45" s="36"/>
+      <c r="E45" s="36"/>
+    </row>
+    <row r="46" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="63"/>
+      <c r="B46" s="57"/>
+      <c r="C46" s="28"/>
+      <c r="D46" s="32"/>
+      <c r="E46" s="32"/>
+    </row>
+    <row r="47" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="63"/>
+      <c r="B47" s="57"/>
+      <c r="C47" s="28"/>
+      <c r="D47" s="32"/>
+      <c r="E47" s="32"/>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A48" s="63"/>
+      <c r="B48" s="57"/>
+      <c r="C48" s="28"/>
+      <c r="D48" s="32"/>
+      <c r="E48" s="32"/>
+    </row>
+    <row r="49" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="61"/>
+      <c r="B49" s="58"/>
+      <c r="C49" s="34"/>
+      <c r="D49" s="37"/>
+      <c r="E49" s="37"/>
+    </row>
+    <row r="50" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B50" s="18"/>
+      <c r="C50" s="64">
+        <f>SUM(C45:C49)</f>
+        <v>0</v>
+      </c>
+      <c r="D50" s="65"/>
+      <c r="E50" s="65"/>
+    </row>
+    <row r="57" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="58" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="44" t="s">
         <v>16</v>
       </c>
-      <c r="B39" s="41"/>
-      <c r="C39" s="2">
+      <c r="B58" s="45"/>
+      <c r="C58" s="2">
         <f>MROUND(SUM(C9,C13,C17,C22,C28,C33,C38) /60,0.2)</f>
         <v>19.600000000000001</v>
       </c>
-      <c r="D39" s="3"/>
-      <c r="E39" s="4"/>
-    </row>
-    <row r="40" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="43" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="44" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="45" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="46" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="47" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="D58" s="3"/>
+      <c r="E58" s="4"/>
+    </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="14">
     <mergeCell ref="B14:B16"/>
-    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="A58:B58"/>
     <mergeCell ref="B10:B12"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
@@ -1578,6 +1734,8 @@
     <mergeCell ref="B23:B27"/>
     <mergeCell ref="B29:B32"/>
     <mergeCell ref="B34:B37"/>
+    <mergeCell ref="B39:B43"/>
+    <mergeCell ref="B45:B49"/>
   </mergeCells>
   <dataValidations disablePrompts="1" count="1">
     <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B6 C6:C8 B10 C10:C12 C16 B14:C14 C20 B18:C18 C25 B23:C23" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
@@ -1617,6 +1775,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010051C931FEC57CD24D841BB655C8BA0DFF" ma:contentTypeVersion="14" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="f47e485f4ad8d247f3dfedaee1362e95">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3eb094ff-ec8d-44d8-be06-94ad3ec8832a" xmlns:ns3="4356f79f-5386-4bda-9d92-82d8bd7b074e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="da34bf24383b1ce13aa9c82f6b8627bb" ns2:_="" ns3:_="">
     <xsd:import namespace="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
@@ -1829,15 +1996,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
   <ds:schemaRefs>
@@ -1856,6 +2014,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5A40649F-4D7C-4B62-9A51-E0A7D9450EFE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1872,12 +2038,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
doc(rapport) ecriture du chapitre sur l'utilisation de l'IA
</commit_message>
<xml_diff>
--- a/doc/JDT-P_OO.xlsx
+++ b/doc/JDT-P_OO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pi46vew\Documents\GitHub\P_OO-ShootMeUp-\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{602A9E34-BAA7-4B82-97A0-94B5873DE484}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{695DED94-BCC1-4F5E-A03D-AC436CAB36AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="76">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -263,6 +263,21 @@
   </si>
   <si>
     <t>Ecriture de RobotTests</t>
+  </si>
+  <si>
+    <t>Diagramme de classe</t>
+  </si>
+  <si>
+    <t>Création du diagramme de classe sur draw.io</t>
+  </si>
+  <si>
+    <t>Ecriture du chapitre sue le diagramme de classe</t>
+  </si>
+  <si>
+    <t>IA</t>
+  </si>
+  <si>
+    <t>Ecriture du chapitre sur l'utilisation de l'IA</t>
   </si>
 </sst>
 </file>
@@ -646,6 +661,23 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -710,23 +742,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1060,10 +1075,10 @@
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="49" t="s">
+      <c r="B1" s="54" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="49"/>
+      <c r="C1" s="54"/>
       <c r="D1" s="8" t="s">
         <v>2</v>
       </c>
@@ -1075,10 +1090,10 @@
       <c r="A2" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="49" t="s">
+      <c r="B2" s="54" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="49"/>
+      <c r="C2" s="54"/>
       <c r="D2" s="8" t="s">
         <v>4</v>
       </c>
@@ -1090,10 +1105,10 @@
       <c r="A3" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="49" t="s">
+      <c r="B3" s="54" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="49"/>
+      <c r="C3" s="54"/>
       <c r="D3" s="8" t="s">
         <v>7</v>
       </c>
@@ -1105,12 +1120,12 @@
       <c r="A4" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="50" t="s">
+      <c r="B4" s="55" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="51"/>
-      <c r="D4" s="51"/>
-      <c r="E4" s="52"/>
+      <c r="C4" s="56"/>
+      <c r="D4" s="56"/>
+      <c r="E4" s="57"/>
     </row>
     <row r="5" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="39" t="s">
@@ -1133,7 +1148,7 @@
       <c r="A6" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="42">
+      <c r="B6" s="47">
         <v>45894</v>
       </c>
       <c r="C6" s="17">
@@ -1150,7 +1165,7 @@
       <c r="A7" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="53"/>
+      <c r="B7" s="58"/>
       <c r="C7" s="9">
         <v>45</v>
       </c>
@@ -1165,7 +1180,7 @@
       <c r="A8" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="54"/>
+      <c r="B8" s="59"/>
       <c r="C8" s="16">
         <v>45</v>
       </c>
@@ -1192,7 +1207,7 @@
       <c r="A10" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="B10" s="46">
+      <c r="B10" s="51">
         <v>46269</v>
       </c>
       <c r="C10" s="17">
@@ -1209,7 +1224,7 @@
       <c r="A11" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="47"/>
+      <c r="B11" s="52"/>
       <c r="C11" s="9">
         <v>120</v>
       </c>
@@ -1224,7 +1239,7 @@
       <c r="A12" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="B12" s="48"/>
+      <c r="B12" s="53"/>
       <c r="C12" s="16">
         <v>15</v>
       </c>
@@ -1251,7 +1266,7 @@
       <c r="A14" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="B14" s="42">
+      <c r="B14" s="47">
         <v>46276</v>
       </c>
       <c r="C14" s="17">
@@ -1268,7 +1283,7 @@
       <c r="A15" s="28" t="s">
         <v>37</v>
       </c>
-      <c r="B15" s="43"/>
+      <c r="B15" s="48"/>
       <c r="C15" s="28">
         <v>20</v>
       </c>
@@ -1281,7 +1296,7 @@
       <c r="A16" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="B16" s="43"/>
+      <c r="B16" s="48"/>
       <c r="C16" s="9">
         <v>10</v>
       </c>
@@ -1306,7 +1321,7 @@
       <c r="A18" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="B18" s="42">
+      <c r="B18" s="47">
         <v>46283</v>
       </c>
       <c r="C18" s="29">
@@ -1321,7 +1336,7 @@
       <c r="A19" s="28" t="s">
         <v>40</v>
       </c>
-      <c r="B19" s="43"/>
+      <c r="B19" s="48"/>
       <c r="C19" s="30">
         <v>40</v>
       </c>
@@ -1334,7 +1349,7 @@
       <c r="A20" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="B20" s="43"/>
+      <c r="B20" s="48"/>
       <c r="C20" s="31">
         <v>30</v>
       </c>
@@ -1347,7 +1362,7 @@
       <c r="A21" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="B21" s="43"/>
+      <c r="B21" s="48"/>
       <c r="C21" s="30">
         <v>60</v>
       </c>
@@ -1372,7 +1387,7 @@
       <c r="A23" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="B23" s="42">
+      <c r="B23" s="47">
         <v>46290</v>
       </c>
       <c r="C23" s="17">
@@ -1387,7 +1402,7 @@
       <c r="A24" s="28" t="s">
         <v>40</v>
       </c>
-      <c r="B24" s="43"/>
+      <c r="B24" s="48"/>
       <c r="C24" s="28">
         <v>20</v>
       </c>
@@ -1400,7 +1415,7 @@
       <c r="A25" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="B25" s="43"/>
+      <c r="B25" s="48"/>
       <c r="C25" s="9">
         <v>25</v>
       </c>
@@ -1413,7 +1428,7 @@
       <c r="A26" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="B26" s="43"/>
+      <c r="B26" s="48"/>
       <c r="C26" s="28">
         <v>60</v>
       </c>
@@ -1426,7 +1441,7 @@
       <c r="A27" s="28" t="s">
         <v>50</v>
       </c>
-      <c r="B27" s="55"/>
+      <c r="B27" s="60"/>
       <c r="C27" s="34">
         <v>30</v>
       </c>
@@ -1451,7 +1466,7 @@
       <c r="A29" s="38" t="s">
         <v>50</v>
       </c>
-      <c r="B29" s="56">
+      <c r="B29" s="61">
         <v>46297</v>
       </c>
       <c r="C29" s="38">
@@ -1466,7 +1481,7 @@
       <c r="A30" s="28" t="s">
         <v>50</v>
       </c>
-      <c r="B30" s="57"/>
+      <c r="B30" s="62"/>
       <c r="C30" s="28">
         <v>45</v>
       </c>
@@ -1479,7 +1494,7 @@
       <c r="A31" s="28" t="s">
         <v>54</v>
       </c>
-      <c r="B31" s="57"/>
+      <c r="B31" s="62"/>
       <c r="C31" s="28">
         <v>60</v>
       </c>
@@ -1492,7 +1507,7 @@
       <c r="A32" s="28" t="s">
         <v>56</v>
       </c>
-      <c r="B32" s="58"/>
+      <c r="B32" s="63"/>
       <c r="C32" s="28">
         <v>30</v>
       </c>
@@ -1517,7 +1532,7 @@
       <c r="A34" s="38" t="s">
         <v>58</v>
       </c>
-      <c r="B34" s="56">
+      <c r="B34" s="61">
         <v>46304</v>
       </c>
       <c r="C34" s="38">
@@ -1532,7 +1547,7 @@
       <c r="A35" s="28" t="s">
         <v>60</v>
       </c>
-      <c r="B35" s="59"/>
+      <c r="B35" s="64"/>
       <c r="C35" s="28">
         <v>50</v>
       </c>
@@ -1545,7 +1560,7 @@
       <c r="A36" s="28" t="s">
         <v>60</v>
       </c>
-      <c r="B36" s="59"/>
+      <c r="B36" s="64"/>
       <c r="C36" s="28">
         <v>45</v>
       </c>
@@ -1558,7 +1573,7 @@
       <c r="A37" s="34" t="s">
         <v>64</v>
       </c>
-      <c r="B37" s="60"/>
+      <c r="B37" s="65"/>
       <c r="C37" s="34">
         <v>25</v>
       </c>
@@ -1580,10 +1595,10 @@
       <c r="E38" s="18"/>
     </row>
     <row r="39" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="62" t="s">
+      <c r="A39" s="43" t="s">
         <v>64</v>
       </c>
-      <c r="B39" s="56">
+      <c r="B39" s="61">
         <v>46318</v>
       </c>
       <c r="C39" s="38">
@@ -1595,10 +1610,10 @@
       <c r="E39" s="36"/>
     </row>
     <row r="40" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="63" t="s">
+      <c r="A40" s="44" t="s">
         <v>66</v>
       </c>
-      <c r="B40" s="57"/>
+      <c r="B40" s="62"/>
       <c r="C40" s="28">
         <v>20</v>
       </c>
@@ -1608,10 +1623,10 @@
       <c r="E40" s="32"/>
     </row>
     <row r="41" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="63" t="s">
+      <c r="A41" s="44" t="s">
         <v>66</v>
       </c>
-      <c r="B41" s="57"/>
+      <c r="B41" s="62"/>
       <c r="C41" s="28">
         <v>40</v>
       </c>
@@ -1621,10 +1636,10 @@
       <c r="E41" s="32"/>
     </row>
     <row r="42" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="63" t="s">
+      <c r="A42" s="44" t="s">
         <v>66</v>
       </c>
-      <c r="B42" s="57"/>
+      <c r="B42" s="62"/>
       <c r="C42" s="28">
         <v>30</v>
       </c>
@@ -1634,10 +1649,10 @@
       <c r="E42" s="32"/>
     </row>
     <row r="43" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="61" t="s">
+      <c r="A43" s="42" t="s">
         <v>66</v>
       </c>
-      <c r="B43" s="58"/>
+      <c r="B43" s="63"/>
       <c r="C43" s="34">
         <v>30</v>
       </c>
@@ -1651,46 +1666,64 @@
         <v>15</v>
       </c>
       <c r="B44" s="18"/>
-      <c r="C44" s="64">
+      <c r="C44" s="45">
         <f>SUM(C39:C43)</f>
         <v>180</v>
       </c>
-      <c r="D44" s="65"/>
-      <c r="E44" s="65"/>
+      <c r="D44" s="46"/>
+      <c r="E44" s="46"/>
     </row>
     <row r="45" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="62"/>
-      <c r="B45" s="56">
+      <c r="A45" s="43" t="s">
+        <v>71</v>
+      </c>
+      <c r="B45" s="61">
         <v>46325</v>
       </c>
-      <c r="C45" s="38"/>
-      <c r="D45" s="36"/>
+      <c r="C45" s="38">
+        <v>50</v>
+      </c>
+      <c r="D45" s="36" t="s">
+        <v>72</v>
+      </c>
       <c r="E45" s="36"/>
     </row>
     <row r="46" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="63"/>
-      <c r="B46" s="57"/>
-      <c r="C46" s="28"/>
-      <c r="D46" s="32"/>
+      <c r="A46" s="44" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46" s="62"/>
+      <c r="C46" s="28">
+        <v>40</v>
+      </c>
+      <c r="D46" s="32" t="s">
+        <v>73</v>
+      </c>
       <c r="E46" s="32"/>
     </row>
     <row r="47" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="63"/>
-      <c r="B47" s="57"/>
-      <c r="C47" s="28"/>
-      <c r="D47" s="32"/>
+      <c r="A47" s="44" t="s">
+        <v>74</v>
+      </c>
+      <c r="B47" s="62"/>
+      <c r="C47" s="28">
+        <v>60</v>
+      </c>
+      <c r="D47" s="32" t="s">
+        <v>75</v>
+      </c>
       <c r="E47" s="32"/>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A48" s="63"/>
-      <c r="B48" s="57"/>
+      <c r="A48" s="44"/>
+      <c r="B48" s="62"/>
       <c r="C48" s="28"/>
       <c r="D48" s="32"/>
       <c r="E48" s="32"/>
     </row>
     <row r="49" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="61"/>
-      <c r="B49" s="58"/>
+      <c r="A49" s="42"/>
+      <c r="B49" s="63"/>
       <c r="C49" s="34"/>
       <c r="D49" s="37"/>
       <c r="E49" s="37"/>
@@ -1700,19 +1733,19 @@
         <v>15</v>
       </c>
       <c r="B50" s="18"/>
-      <c r="C50" s="64">
+      <c r="C50" s="45">
         <f>SUM(C45:C49)</f>
-        <v>0</v>
-      </c>
-      <c r="D50" s="65"/>
-      <c r="E50" s="65"/>
+        <v>150</v>
+      </c>
+      <c r="D50" s="46"/>
+      <c r="E50" s="46"/>
     </row>
     <row r="57" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="58" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="44" t="s">
+      <c r="A58" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="B58" s="45"/>
+      <c r="B58" s="50"/>
       <c r="C58" s="2">
         <f>MROUND(SUM(C9,C13,C17,C22,C28,C33,C38) /60,0.2)</f>
         <v>19.600000000000001</v>
@@ -1775,15 +1808,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010051C931FEC57CD24D841BB655C8BA0DFF" ma:contentTypeVersion="14" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="f47e485f4ad8d247f3dfedaee1362e95">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3eb094ff-ec8d-44d8-be06-94ad3ec8832a" xmlns:ns3="4356f79f-5386-4bda-9d92-82d8bd7b074e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="da34bf24383b1ce13aa9c82f6b8627bb" ns2:_="" ns3:_="">
     <xsd:import namespace="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
@@ -1996,6 +2020,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
   <ds:schemaRefs>
@@ -2014,14 +2047,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5A40649F-4D7C-4B62-9A51-E0A7D9450EFE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2038,4 +2063,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
chore(JDT) mise à jour du cahier des charges
</commit_message>
<xml_diff>
--- a/doc/JDT-P_OO.xlsx
+++ b/doc/JDT-P_OO.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pi46vew\Documents\GitHub\P_OO-ShootMeUp-\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{695DED94-BCC1-4F5E-A03D-AC436CAB36AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{527F5977-349B-48C9-A7A1-52DAD7CC326C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$58</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$51</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="79">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -187,69 +187,27 @@
     <t>Instantiation du burger sur la carte lors du clique mais pas réussi à ajouter la trajectoire (User Story num 2)</t>
   </si>
   <si>
-    <t>Les attauques burger vont en direction de la souris</t>
-  </si>
-  <si>
-    <t>Ajout d'un cooldown aux tirs burger</t>
-  </si>
-  <si>
-    <t>les burgers sont detruit si ils touches les bords du gamespace</t>
-  </si>
-  <si>
     <t>Attaque mélée</t>
   </si>
   <si>
-    <t>Ajout d'une attaque d'un mode "mélée" pour le joueur quand il fait une attaque mélée</t>
-  </si>
-  <si>
     <t>Manager</t>
   </si>
   <si>
-    <t>Commencer l'ajout d'un enemie de type Manager. Création de la classe et des premiers attributs</t>
-  </si>
-  <si>
-    <t>Ajout d'un déplacement aléatoire des managers</t>
-  </si>
-  <si>
-    <t>Ajout d'une barre de vie au manager</t>
-  </si>
-  <si>
     <t>barre de vie</t>
   </si>
   <si>
-    <t>Création d'une barre de vie et d un écran de mort quand les PV passe à 0</t>
-  </si>
-  <si>
     <t>barre d'argent</t>
   </si>
   <si>
-    <t>Commencer la création d'une barre d'argent pour pouvoir gagner</t>
-  </si>
-  <si>
     <t>Robot</t>
   </si>
   <si>
-    <t>Création d'un ennemi robot en s'inspirant beacoup de l'ennemi manager</t>
-  </si>
-  <si>
     <t>Faisceau</t>
   </si>
   <si>
-    <t>Création d'un faisceau pouvant aller dans les quatres direction</t>
-  </si>
-  <si>
-    <t>Fait en sorte que les faisceaux fassent des dégats quand ils touches le joueur et qu'ils soit tirés par les robots</t>
-  </si>
-  <si>
-    <t>Commencer la création des obstacles</t>
-  </si>
-  <si>
     <t>Obstacle</t>
   </si>
   <si>
-    <t>Finis la création des obstacles et fait en sorte que les Manager et Robot trouve un nouveau chemin</t>
-  </si>
-  <si>
     <t>Tests</t>
   </si>
   <si>
@@ -278,6 +236,57 @@
   </si>
   <si>
     <t>Ecriture du chapitre sur l'utilisation de l'IA</t>
+  </si>
+  <si>
+    <t>Les attauques burger vont en direction de la souris (US 2)</t>
+  </si>
+  <si>
+    <t>Ajout d'un cooldown aux tirs burger (US 2)</t>
+  </si>
+  <si>
+    <t>les burgers sont detruit si ils touches les bords du gamespace (US 2)</t>
+  </si>
+  <si>
+    <t>Ajout d'une attaque d'un mode "mélée" pour le joueur quand il fait une attaque mélée (US 3)</t>
+  </si>
+  <si>
+    <t>Commencer l'ajout d'un enemie de type Manager. Création de la classe et des premiers attributs (US 4)</t>
+  </si>
+  <si>
+    <t>Ajout d'un déplacement aléatoire des managers (US 4)</t>
+  </si>
+  <si>
+    <t>Ajout d'une barre de vie au manager (US 4)</t>
+  </si>
+  <si>
+    <t>Création d'une barre de vie et d un écran de mort quand les PV passe à 0 (US 8)</t>
+  </si>
+  <si>
+    <t>Commencer la création d'une barre d'argent pour pouvoir gagner (US 9)</t>
+  </si>
+  <si>
+    <t>Création d'un ennemi robot en s'inspirant beacoup de l'ennemi manager (US 5)</t>
+  </si>
+  <si>
+    <t>Création d'un faisceau pouvant aller dans les quatres direction (US 6)</t>
+  </si>
+  <si>
+    <t>Fait en sorte que les faisceaux fassent des dégats quand ils touches le joueur et qu'ils soit tirés par les robots (US 6)</t>
+  </si>
+  <si>
+    <t>Commencer la création des obstacles (US 10)</t>
+  </si>
+  <si>
+    <t>Finis la création des obstacles et fait en sorte que les Manager et Robot trouve un nouveau chemin (US 10)</t>
+  </si>
+  <si>
+    <t>Bilan et Conclusion</t>
+  </si>
+  <si>
+    <t>Ecriture des chapitre "Bilan du déroulement du projet" , "Bilan produit", "Conclusion personnelle"</t>
+  </si>
+  <si>
+    <t>Ecriture de 6 tests supplémentaire et rendu du projet</t>
   </si>
 </sst>
 </file>
@@ -1059,7 +1068,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E58"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33" style="1" customWidth="1"/>
@@ -1394,7 +1403,7 @@
         <v>45</v>
       </c>
       <c r="D23" s="19" t="s">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="E23" s="22"/>
     </row>
@@ -1407,7 +1416,7 @@
         <v>20</v>
       </c>
       <c r="D24" s="32" t="s">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="E24" s="23"/>
     </row>
@@ -1420,33 +1429,33 @@
         <v>25</v>
       </c>
       <c r="D25" s="20" t="s">
-        <v>47</v>
+        <v>64</v>
       </c>
       <c r="E25" s="23"/>
     </row>
     <row r="26" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="12" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B26" s="48"/>
       <c r="C26" s="28">
         <v>60</v>
       </c>
       <c r="D26" s="32" t="s">
-        <v>49</v>
+        <v>65</v>
       </c>
       <c r="E26" s="32"/>
     </row>
     <row r="27" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="28" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B27" s="60"/>
       <c r="C27" s="34">
         <v>30</v>
       </c>
       <c r="D27" s="35" t="s">
-        <v>51</v>
+        <v>66</v>
       </c>
       <c r="E27" s="34"/>
     </row>
@@ -1464,7 +1473,7 @@
     </row>
     <row r="29" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="38" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B29" s="61">
         <v>46297</v>
@@ -1473,46 +1482,46 @@
         <v>45</v>
       </c>
       <c r="D29" s="36" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
       <c r="E29" s="36"/>
     </row>
     <row r="30" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="28" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B30" s="62"/>
       <c r="C30" s="28">
         <v>45</v>
       </c>
       <c r="D30" s="32" t="s">
-        <v>53</v>
+        <v>68</v>
       </c>
       <c r="E30" s="32"/>
     </row>
     <row r="31" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="28" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="B31" s="62"/>
       <c r="C31" s="28">
         <v>60</v>
       </c>
       <c r="D31" s="32" t="s">
-        <v>55</v>
+        <v>69</v>
       </c>
       <c r="E31" s="32"/>
     </row>
     <row r="32" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="28" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="B32" s="63"/>
       <c r="C32" s="28">
         <v>30</v>
       </c>
       <c r="D32" s="32" t="s">
-        <v>57</v>
+        <v>70</v>
       </c>
       <c r="E32" s="32"/>
     </row>
@@ -1530,7 +1539,7 @@
     </row>
     <row r="34" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="38" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="B34" s="61">
         <v>46304</v>
@@ -1539,46 +1548,46 @@
         <v>60</v>
       </c>
       <c r="D34" s="36" t="s">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="E34" s="36"/>
     </row>
     <row r="35" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="28" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="B35" s="64"/>
       <c r="C35" s="28">
         <v>50</v>
       </c>
       <c r="D35" s="32" t="s">
-        <v>61</v>
+        <v>72</v>
       </c>
       <c r="E35" s="32"/>
     </row>
     <row r="36" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="28" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="B36" s="64"/>
       <c r="C36" s="28">
         <v>45</v>
       </c>
       <c r="D36" s="32" t="s">
-        <v>62</v>
+        <v>73</v>
       </c>
       <c r="E36" s="32"/>
     </row>
     <row r="37" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="34" t="s">
-        <v>64</v>
+        <v>51</v>
       </c>
       <c r="B37" s="65"/>
       <c r="C37" s="34">
         <v>25</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>63</v>
+        <v>74</v>
       </c>
       <c r="E37" s="37"/>
     </row>
@@ -1596,7 +1605,7 @@
     </row>
     <row r="39" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="43" t="s">
-        <v>64</v>
+        <v>51</v>
       </c>
       <c r="B39" s="61">
         <v>46318</v>
@@ -1605,59 +1614,59 @@
         <v>60</v>
       </c>
       <c r="D39" s="36" t="s">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="E39" s="36"/>
     </row>
     <row r="40" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="44" t="s">
-        <v>66</v>
+        <v>52</v>
       </c>
       <c r="B40" s="62"/>
       <c r="C40" s="28">
         <v>20</v>
       </c>
       <c r="D40" s="32" t="s">
-        <v>67</v>
+        <v>53</v>
       </c>
       <c r="E40" s="32"/>
     </row>
     <row r="41" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="44" t="s">
-        <v>66</v>
+        <v>52</v>
       </c>
       <c r="B41" s="62"/>
       <c r="C41" s="28">
         <v>40</v>
       </c>
       <c r="D41" s="32" t="s">
-        <v>68</v>
+        <v>54</v>
       </c>
       <c r="E41" s="32"/>
     </row>
     <row r="42" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="44" t="s">
-        <v>66</v>
+        <v>52</v>
       </c>
       <c r="B42" s="62"/>
       <c r="C42" s="28">
         <v>30</v>
       </c>
       <c r="D42" s="32" t="s">
-        <v>69</v>
+        <v>55</v>
       </c>
       <c r="E42" s="32"/>
     </row>
     <row r="43" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="42" t="s">
-        <v>66</v>
+        <v>52</v>
       </c>
       <c r="B43" s="63"/>
       <c r="C43" s="34">
         <v>30</v>
       </c>
       <c r="D43" s="37" t="s">
-        <v>70</v>
+        <v>56</v>
       </c>
       <c r="E43" s="37"/>
     </row>
@@ -1675,7 +1684,7 @@
     </row>
     <row r="45" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="43" t="s">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="B45" s="61">
         <v>46325</v>
@@ -1684,48 +1693,60 @@
         <v>50</v>
       </c>
       <c r="D45" s="36" t="s">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="E45" s="36"/>
     </row>
     <row r="46" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="44" t="s">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="B46" s="62"/>
       <c r="C46" s="28">
         <v>40</v>
       </c>
       <c r="D46" s="32" t="s">
-        <v>73</v>
+        <v>59</v>
       </c>
       <c r="E46" s="32"/>
     </row>
     <row r="47" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="44" t="s">
-        <v>74</v>
+        <v>60</v>
       </c>
       <c r="B47" s="62"/>
       <c r="C47" s="28">
         <v>60</v>
       </c>
       <c r="D47" s="32" t="s">
-        <v>75</v>
+        <v>61</v>
       </c>
       <c r="E47" s="32"/>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A48" s="44"/>
+      <c r="A48" s="44" t="s">
+        <v>76</v>
+      </c>
       <c r="B48" s="62"/>
-      <c r="C48" s="28"/>
-      <c r="D48" s="32"/>
+      <c r="C48" s="28">
+        <v>60</v>
+      </c>
+      <c r="D48" s="32" t="s">
+        <v>77</v>
+      </c>
       <c r="E48" s="32"/>
     </row>
     <row r="49" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="42"/>
+      <c r="A49" s="42" t="s">
+        <v>52</v>
+      </c>
       <c r="B49" s="63"/>
-      <c r="C49" s="34"/>
-      <c r="D49" s="37"/>
+      <c r="C49" s="34">
+        <v>60</v>
+      </c>
+      <c r="D49" s="37" t="s">
+        <v>78</v>
+      </c>
       <c r="E49" s="37"/>
     </row>
     <row r="50" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -1735,28 +1756,27 @@
       <c r="B50" s="18"/>
       <c r="C50" s="45">
         <f>SUM(C45:C49)</f>
-        <v>150</v>
+        <v>270</v>
       </c>
       <c r="D50" s="46"/>
       <c r="E50" s="46"/>
     </row>
-    <row r="57" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="58" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="49" t="s">
+    <row r="51" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="B58" s="50"/>
-      <c r="C58" s="2">
-        <f>MROUND(SUM(C9,C13,C17,C22,C28,C33,C38) /60,0.2)</f>
-        <v>19.600000000000001</v>
-      </c>
-      <c r="D58" s="3"/>
-      <c r="E58" s="4"/>
+      <c r="B51" s="50"/>
+      <c r="C51" s="2">
+        <f>MROUND(SUM(C9,C13,C17,C22,C28,C33,C38,C44,C50) /60,0.2)</f>
+        <v>27</v>
+      </c>
+      <c r="D51" s="3"/>
+      <c r="E51" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="14">
     <mergeCell ref="B14:B16"/>
-    <mergeCell ref="A58:B58"/>
+    <mergeCell ref="A51:B51"/>
     <mergeCell ref="B10:B12"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
@@ -1770,7 +1790,7 @@
     <mergeCell ref="B39:B43"/>
     <mergeCell ref="B45:B49"/>
   </mergeCells>
-  <dataValidations disablePrompts="1" count="1">
+  <dataValidations count="1">
     <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B6 C6:C8 B10 C10:C12 C16 B14:C14 C20 B18:C18 C25 B23:C23" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
       <formula1>0</formula1>
     </dataValidation>

</xml_diff>

<commit_message>
doc(rapport/JDT) exportation du JDT et du Rapport
</commit_message>
<xml_diff>
--- a/doc/JDT-P_OO.xlsx
+++ b/doc/JDT-P_OO.xlsx
@@ -5,12 +5,12 @@
   <workbookPr updateLinks="never" codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pi46vew\Documents\GitHub\P_OO-ShootMeUp-\doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anton\Documents\GitHub\P_OO-ShootMeUp\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{527F5977-349B-48C9-A7A1-52DAD7CC326C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88BEE98E-84D0-4A51-928D-BCB75F64C8D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="1575" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
@@ -293,7 +293,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Century Gothic"/>
@@ -329,14 +329,6 @@
       <name val="Century Gothic"/>
       <family val="2"/>
     </font>
-    <font>
-      <u/>
-      <sz val="10"/>
-      <color theme="10"/>
-      <name val="Century Gothic"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -516,16 +508,19 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -670,15 +665,6 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -687,10 +673,6 @@
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -753,9 +735,8 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="3">
-    <cellStyle name="Hyperlink" xfId="2" xr:uid="{00000000-000B-0000-0000-000008000000}"/>
-    <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" xr:uid="{00000000-000B-0000-0000-000008000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1069,709 +1050,709 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:E51"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="33" style="1" customWidth="1"/>
-    <col min="2" max="3" width="14.7109375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="108.28515625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="50.7109375" style="1" customWidth="1"/>
-    <col min="6" max="6" width="19.5703125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="36" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="11.42578125" style="1"/>
+    <col min="1" max="1" width="33" style="2" customWidth="1"/>
+    <col min="2" max="3" width="14.7109375" style="2" customWidth="1"/>
+    <col min="4" max="4" width="108.28515625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="50.7109375" style="2" customWidth="1"/>
+    <col min="6" max="6" width="19.5703125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="36" style="2" customWidth="1"/>
+    <col min="8" max="16384" width="11.42578125" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="54" t="s">
+      <c r="B1" s="51" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="54"/>
-      <c r="D1" s="8" t="s">
+      <c r="C1" s="51"/>
+      <c r="D1" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="7" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="54" t="s">
+      <c r="B2" s="51" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="54"/>
-      <c r="D2" s="8" t="s">
+      <c r="C2" s="51"/>
+      <c r="D2" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="7" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="54" t="s">
+      <c r="B3" s="51" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="54"/>
-      <c r="D3" s="8" t="s">
+      <c r="C3" s="51"/>
+      <c r="D3" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="6" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="15" t="s">
+      <c r="A4" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="55" t="s">
+      <c r="B4" s="52" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="56"/>
-      <c r="D4" s="56"/>
-      <c r="E4" s="57"/>
+      <c r="C4" s="53"/>
+      <c r="D4" s="53"/>
+      <c r="E4" s="54"/>
     </row>
     <row r="5" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="39" t="s">
+      <c r="A5" s="40" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="40" t="s">
+      <c r="B5" s="41" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="40" t="s">
+      <c r="C5" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="40" t="s">
+      <c r="D5" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="41" t="s">
+      <c r="E5" s="42" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="47">
+      <c r="B6" s="1">
         <v>45894</v>
       </c>
-      <c r="C6" s="17">
+      <c r="C6" s="18">
         <v>90</v>
       </c>
-      <c r="D6" s="19" t="s">
+      <c r="D6" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="E6" s="22" t="s">
+      <c r="E6" s="23" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="58"/>
-      <c r="C7" s="9">
+      <c r="B7" s="55"/>
+      <c r="C7" s="10">
         <v>45</v>
       </c>
-      <c r="D7" s="20" t="s">
+      <c r="D7" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="E7" s="23" t="s">
+      <c r="E7" s="24" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="13" t="s">
+      <c r="A8" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="59"/>
-      <c r="C8" s="16">
+      <c r="B8" s="56"/>
+      <c r="C8" s="17">
         <v>45</v>
       </c>
-      <c r="D8" s="21" t="s">
+      <c r="D8" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="E8" s="24" t="s">
+      <c r="E8" s="25" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="14" t="s">
+      <c r="A9" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="18"/>
-      <c r="C9" s="25">
+      <c r="B9" s="19"/>
+      <c r="C9" s="26">
         <f>SUM(C6:C8)</f>
         <v>180</v>
       </c>
-      <c r="D9" s="18"/>
-      <c r="E9" s="18"/>
+      <c r="D9" s="19"/>
+      <c r="E9" s="19"/>
     </row>
     <row r="10" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="11" t="s">
+      <c r="A10" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="B10" s="51">
+      <c r="B10" s="48">
         <v>46269</v>
       </c>
-      <c r="C10" s="17">
+      <c r="C10" s="18">
         <v>45</v>
       </c>
-      <c r="D10" s="19" t="s">
+      <c r="D10" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="E10" s="22" t="s">
+      <c r="E10" s="23" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="12" t="s">
+      <c r="A11" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="52"/>
-      <c r="C11" s="9">
+      <c r="B11" s="49"/>
+      <c r="C11" s="10">
         <v>120</v>
       </c>
-      <c r="D11" s="20" t="s">
+      <c r="D11" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="E11" s="23" t="s">
+      <c r="E11" s="24" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="13" t="s">
+      <c r="A12" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="B12" s="53"/>
-      <c r="C12" s="16">
+      <c r="B12" s="50"/>
+      <c r="C12" s="17">
         <v>15</v>
       </c>
-      <c r="D12" s="21" t="s">
+      <c r="D12" s="22" t="s">
         <v>29</v>
       </c>
-      <c r="E12" s="24" t="s">
+      <c r="E12" s="25" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="10" t="s">
+      <c r="A13" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="18"/>
-      <c r="C13" s="25">
+      <c r="B13" s="19"/>
+      <c r="C13" s="26">
         <f>SUM(C10:C12)</f>
         <v>180</v>
       </c>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="11" t="s">
+      <c r="A14" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="B14" s="47">
+      <c r="B14" s="1">
         <v>46276</v>
       </c>
-      <c r="C14" s="17">
+      <c r="C14" s="18">
         <v>60</v>
       </c>
-      <c r="D14" s="26" t="s">
+      <c r="D14" s="27" t="s">
         <v>34</v>
       </c>
-      <c r="E14" s="22" t="s">
+      <c r="E14" s="23" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="28" t="s">
+      <c r="A15" s="29" t="s">
         <v>37</v>
       </c>
-      <c r="B15" s="48"/>
-      <c r="C15" s="28">
+      <c r="B15" s="45"/>
+      <c r="C15" s="29">
         <v>20</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="D15" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="E15" s="23"/>
+      <c r="E15" s="24"/>
     </row>
     <row r="16" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="12" t="s">
+      <c r="A16" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="B16" s="48"/>
-      <c r="C16" s="9">
+      <c r="B16" s="45"/>
+      <c r="C16" s="10">
         <v>10</v>
       </c>
-      <c r="D16" s="27" t="s">
+      <c r="D16" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="E16" s="23"/>
+      <c r="E16" s="24"/>
     </row>
     <row r="17" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="10" t="s">
+      <c r="A17" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="33"/>
-      <c r="C17" s="25">
+      <c r="B17" s="34"/>
+      <c r="C17" s="26">
         <f>SUM(C14:C16)</f>
         <v>90</v>
       </c>
-      <c r="D17" s="18"/>
-      <c r="E17" s="18"/>
+      <c r="D17" s="19"/>
+      <c r="E17" s="19"/>
     </row>
     <row r="18" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="11" t="s">
+      <c r="A18" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="B18" s="47">
+      <c r="B18" s="1">
         <v>46283</v>
       </c>
-      <c r="C18" s="29">
+      <c r="C18" s="30">
         <v>50</v>
       </c>
-      <c r="D18" s="19" t="s">
+      <c r="D18" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="E18" s="22"/>
+      <c r="E18" s="23"/>
     </row>
     <row r="19" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="28" t="s">
+      <c r="A19" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="B19" s="48"/>
-      <c r="C19" s="30">
+      <c r="B19" s="45"/>
+      <c r="C19" s="31">
         <v>40</v>
       </c>
-      <c r="D19" s="32" t="s">
+      <c r="D19" s="33" t="s">
         <v>42</v>
       </c>
-      <c r="E19" s="23"/>
+      <c r="E19" s="24"/>
     </row>
     <row r="20" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="12" t="s">
+      <c r="A20" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="B20" s="48"/>
-      <c r="C20" s="31">
+      <c r="B20" s="45"/>
+      <c r="C20" s="32">
         <v>30</v>
       </c>
-      <c r="D20" s="20" t="s">
+      <c r="D20" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="E20" s="23"/>
+      <c r="E20" s="24"/>
     </row>
     <row r="21" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="12" t="s">
+      <c r="A21" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="B21" s="48"/>
-      <c r="C21" s="30">
+      <c r="B21" s="45"/>
+      <c r="C21" s="31">
         <v>60</v>
       </c>
-      <c r="D21" s="32" t="s">
+      <c r="D21" s="33" t="s">
         <v>44</v>
       </c>
-      <c r="E21" s="32"/>
+      <c r="E21" s="33"/>
     </row>
     <row r="22" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="10" t="s">
+      <c r="A22" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="B22" s="18"/>
-      <c r="C22" s="25">
+      <c r="B22" s="19"/>
+      <c r="C22" s="26">
         <f>SUM(C18:C21)</f>
         <v>180</v>
       </c>
-      <c r="D22" s="18"/>
-      <c r="E22" s="18"/>
+      <c r="D22" s="19"/>
+      <c r="E22" s="19"/>
     </row>
     <row r="23" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="11" t="s">
+      <c r="A23" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="B23" s="47">
+      <c r="B23" s="1">
         <v>46290</v>
       </c>
-      <c r="C23" s="17">
+      <c r="C23" s="18">
         <v>45</v>
       </c>
-      <c r="D23" s="19" t="s">
+      <c r="D23" s="20" t="s">
         <v>62</v>
       </c>
-      <c r="E23" s="22"/>
+      <c r="E23" s="23"/>
     </row>
     <row r="24" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="28" t="s">
+      <c r="A24" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="B24" s="48"/>
-      <c r="C24" s="28">
+      <c r="B24" s="45"/>
+      <c r="C24" s="29">
         <v>20</v>
       </c>
-      <c r="D24" s="32" t="s">
+      <c r="D24" s="33" t="s">
         <v>63</v>
       </c>
-      <c r="E24" s="23"/>
+      <c r="E24" s="24"/>
     </row>
     <row r="25" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="12" t="s">
+      <c r="A25" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="B25" s="48"/>
-      <c r="C25" s="9">
+      <c r="B25" s="45"/>
+      <c r="C25" s="10">
         <v>25</v>
       </c>
-      <c r="D25" s="20" t="s">
+      <c r="D25" s="21" t="s">
         <v>64</v>
       </c>
-      <c r="E25" s="23"/>
+      <c r="E25" s="24"/>
     </row>
     <row r="26" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="12" t="s">
+      <c r="A26" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="B26" s="48"/>
-      <c r="C26" s="28">
+      <c r="B26" s="45"/>
+      <c r="C26" s="29">
         <v>60</v>
       </c>
-      <c r="D26" s="32" t="s">
+      <c r="D26" s="33" t="s">
         <v>65</v>
       </c>
-      <c r="E26" s="32"/>
+      <c r="E26" s="33"/>
     </row>
     <row r="27" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="28" t="s">
+      <c r="A27" s="29" t="s">
         <v>46</v>
       </c>
-      <c r="B27" s="60"/>
-      <c r="C27" s="34">
+      <c r="B27" s="57"/>
+      <c r="C27" s="35">
         <v>30</v>
       </c>
-      <c r="D27" s="35" t="s">
+      <c r="D27" s="36" t="s">
         <v>66</v>
       </c>
-      <c r="E27" s="34"/>
+      <c r="E27" s="35"/>
     </row>
     <row r="28" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="10" t="s">
+      <c r="A28" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="B28" s="18"/>
-      <c r="C28" s="25">
+      <c r="B28" s="19"/>
+      <c r="C28" s="26">
         <f>SUM(C23:C27)</f>
         <v>180</v>
       </c>
-      <c r="D28" s="18"/>
-      <c r="E28" s="18"/>
+      <c r="D28" s="19"/>
+      <c r="E28" s="19"/>
     </row>
     <row r="29" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="38" t="s">
+      <c r="A29" s="39" t="s">
         <v>46</v>
       </c>
-      <c r="B29" s="61">
+      <c r="B29" s="58">
         <v>46297</v>
       </c>
-      <c r="C29" s="38">
+      <c r="C29" s="39">
         <v>45</v>
       </c>
-      <c r="D29" s="36" t="s">
+      <c r="D29" s="37" t="s">
         <v>67</v>
       </c>
-      <c r="E29" s="36"/>
+      <c r="E29" s="37"/>
     </row>
     <row r="30" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="28" t="s">
+      <c r="A30" s="29" t="s">
         <v>46</v>
       </c>
-      <c r="B30" s="62"/>
-      <c r="C30" s="28">
+      <c r="B30" s="59"/>
+      <c r="C30" s="29">
         <v>45</v>
       </c>
-      <c r="D30" s="32" t="s">
+      <c r="D30" s="33" t="s">
         <v>68</v>
       </c>
-      <c r="E30" s="32"/>
+      <c r="E30" s="33"/>
     </row>
     <row r="31" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="28" t="s">
+      <c r="A31" s="29" t="s">
         <v>47</v>
       </c>
-      <c r="B31" s="62"/>
-      <c r="C31" s="28">
+      <c r="B31" s="59"/>
+      <c r="C31" s="29">
         <v>60</v>
       </c>
-      <c r="D31" s="32" t="s">
+      <c r="D31" s="33" t="s">
         <v>69</v>
       </c>
-      <c r="E31" s="32"/>
+      <c r="E31" s="33"/>
     </row>
     <row r="32" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="28" t="s">
+      <c r="A32" s="29" t="s">
         <v>48</v>
       </c>
-      <c r="B32" s="63"/>
-      <c r="C32" s="28">
+      <c r="B32" s="60"/>
+      <c r="C32" s="29">
         <v>30</v>
       </c>
-      <c r="D32" s="32" t="s">
+      <c r="D32" s="33" t="s">
         <v>70</v>
       </c>
-      <c r="E32" s="32"/>
+      <c r="E32" s="33"/>
     </row>
     <row r="33" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="10" t="s">
+      <c r="A33" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="18"/>
-      <c r="C33" s="25">
+      <c r="B33" s="19"/>
+      <c r="C33" s="26">
         <f>SUM(C29:C32)</f>
         <v>180</v>
       </c>
-      <c r="D33" s="18"/>
-      <c r="E33" s="18"/>
+      <c r="D33" s="19"/>
+      <c r="E33" s="19"/>
     </row>
     <row r="34" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="38" t="s">
+      <c r="A34" s="39" t="s">
         <v>49</v>
       </c>
-      <c r="B34" s="61">
+      <c r="B34" s="58">
         <v>46304</v>
       </c>
-      <c r="C34" s="38">
+      <c r="C34" s="39">
         <v>60</v>
       </c>
-      <c r="D34" s="36" t="s">
+      <c r="D34" s="37" t="s">
         <v>71</v>
       </c>
-      <c r="E34" s="36"/>
+      <c r="E34" s="37"/>
     </row>
     <row r="35" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="28" t="s">
+      <c r="A35" s="29" t="s">
         <v>50</v>
       </c>
-      <c r="B35" s="64"/>
-      <c r="C35" s="28">
+      <c r="B35" s="61"/>
+      <c r="C35" s="29">
         <v>50</v>
       </c>
-      <c r="D35" s="32" t="s">
+      <c r="D35" s="33" t="s">
         <v>72</v>
       </c>
-      <c r="E35" s="32"/>
+      <c r="E35" s="33"/>
     </row>
     <row r="36" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="28" t="s">
+      <c r="A36" s="29" t="s">
         <v>50</v>
       </c>
-      <c r="B36" s="64"/>
-      <c r="C36" s="28">
+      <c r="B36" s="61"/>
+      <c r="C36" s="29">
         <v>45</v>
       </c>
-      <c r="D36" s="32" t="s">
+      <c r="D36" s="33" t="s">
         <v>73</v>
       </c>
-      <c r="E36" s="32"/>
+      <c r="E36" s="33"/>
     </row>
     <row r="37" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="34" t="s">
+      <c r="A37" s="35" t="s">
         <v>51</v>
       </c>
-      <c r="B37" s="65"/>
-      <c r="C37" s="34">
+      <c r="B37" s="62"/>
+      <c r="C37" s="35">
         <v>25</v>
       </c>
-      <c r="D37" s="1" t="s">
+      <c r="D37" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="E37" s="37"/>
+      <c r="E37" s="38"/>
     </row>
     <row r="38" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="10" t="s">
+      <c r="A38" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="B38" s="18"/>
-      <c r="C38" s="25">
+      <c r="B38" s="19"/>
+      <c r="C38" s="26">
         <f>SUM(C34:C37)</f>
         <v>180</v>
       </c>
-      <c r="D38" s="18"/>
-      <c r="E38" s="18"/>
+      <c r="D38" s="19"/>
+      <c r="E38" s="19"/>
     </row>
     <row r="39" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="43" t="s">
+      <c r="A39" s="39" t="s">
         <v>51</v>
       </c>
-      <c r="B39" s="61">
+      <c r="B39" s="58">
         <v>46318</v>
       </c>
-      <c r="C39" s="38">
+      <c r="C39" s="39">
         <v>60</v>
       </c>
-      <c r="D39" s="36" t="s">
+      <c r="D39" s="37" t="s">
         <v>75</v>
       </c>
-      <c r="E39" s="36"/>
+      <c r="E39" s="37"/>
     </row>
     <row r="40" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="44" t="s">
+      <c r="A40" s="29" t="s">
         <v>52</v>
       </c>
-      <c r="B40" s="62"/>
-      <c r="C40" s="28">
+      <c r="B40" s="59"/>
+      <c r="C40" s="29">
         <v>20</v>
       </c>
-      <c r="D40" s="32" t="s">
+      <c r="D40" s="33" t="s">
         <v>53</v>
       </c>
-      <c r="E40" s="32"/>
+      <c r="E40" s="33"/>
     </row>
     <row r="41" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="44" t="s">
+      <c r="A41" s="29" t="s">
         <v>52</v>
       </c>
-      <c r="B41" s="62"/>
-      <c r="C41" s="28">
+      <c r="B41" s="59"/>
+      <c r="C41" s="29">
         <v>40</v>
       </c>
-      <c r="D41" s="32" t="s">
+      <c r="D41" s="33" t="s">
         <v>54</v>
       </c>
-      <c r="E41" s="32"/>
+      <c r="E41" s="33"/>
     </row>
     <row r="42" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="44" t="s">
+      <c r="A42" s="29" t="s">
         <v>52</v>
       </c>
-      <c r="B42" s="62"/>
-      <c r="C42" s="28">
+      <c r="B42" s="59"/>
+      <c r="C42" s="29">
         <v>30</v>
       </c>
-      <c r="D42" s="32" t="s">
+      <c r="D42" s="33" t="s">
         <v>55</v>
       </c>
-      <c r="E42" s="32"/>
+      <c r="E42" s="33"/>
     </row>
     <row r="43" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="42" t="s">
+      <c r="A43" s="35" t="s">
         <v>52</v>
       </c>
-      <c r="B43" s="63"/>
-      <c r="C43" s="34">
+      <c r="B43" s="60"/>
+      <c r="C43" s="35">
         <v>30</v>
       </c>
-      <c r="D43" s="37" t="s">
+      <c r="D43" s="38" t="s">
         <v>56</v>
       </c>
-      <c r="E43" s="37"/>
+      <c r="E43" s="38"/>
     </row>
     <row r="44" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="10" t="s">
+      <c r="A44" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="B44" s="18"/>
-      <c r="C44" s="45">
+      <c r="B44" s="19"/>
+      <c r="C44" s="43">
         <f>SUM(C39:C43)</f>
         <v>180</v>
       </c>
-      <c r="D44" s="46"/>
-      <c r="E44" s="46"/>
+      <c r="D44" s="44"/>
+      <c r="E44" s="44"/>
     </row>
     <row r="45" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="43" t="s">
+      <c r="A45" s="39" t="s">
         <v>57</v>
       </c>
-      <c r="B45" s="61">
+      <c r="B45" s="58">
         <v>46325</v>
       </c>
-      <c r="C45" s="38">
+      <c r="C45" s="39">
         <v>50</v>
       </c>
-      <c r="D45" s="36" t="s">
+      <c r="D45" s="37" t="s">
         <v>58</v>
       </c>
-      <c r="E45" s="36"/>
+      <c r="E45" s="37"/>
     </row>
     <row r="46" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="44" t="s">
+      <c r="A46" s="29" t="s">
         <v>57</v>
       </c>
-      <c r="B46" s="62"/>
-      <c r="C46" s="28">
+      <c r="B46" s="59"/>
+      <c r="C46" s="29">
         <v>40</v>
       </c>
-      <c r="D46" s="32" t="s">
+      <c r="D46" s="33" t="s">
         <v>59</v>
       </c>
-      <c r="E46" s="32"/>
+      <c r="E46" s="33"/>
     </row>
     <row r="47" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="44" t="s">
+      <c r="A47" s="29" t="s">
         <v>60</v>
       </c>
-      <c r="B47" s="62"/>
-      <c r="C47" s="28">
+      <c r="B47" s="59"/>
+      <c r="C47" s="29">
         <v>60</v>
       </c>
-      <c r="D47" s="32" t="s">
+      <c r="D47" s="33" t="s">
         <v>61</v>
       </c>
-      <c r="E47" s="32"/>
+      <c r="E47" s="33"/>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A48" s="44" t="s">
+      <c r="A48" s="29" t="s">
         <v>76</v>
       </c>
-      <c r="B48" s="62"/>
-      <c r="C48" s="28">
+      <c r="B48" s="59"/>
+      <c r="C48" s="29">
         <v>60</v>
       </c>
-      <c r="D48" s="32" t="s">
+      <c r="D48" s="33" t="s">
         <v>77</v>
       </c>
-      <c r="E48" s="32"/>
+      <c r="E48" s="33"/>
     </row>
     <row r="49" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="42" t="s">
+      <c r="A49" s="35" t="s">
         <v>52</v>
       </c>
-      <c r="B49" s="63"/>
-      <c r="C49" s="34">
+      <c r="B49" s="60"/>
+      <c r="C49" s="35">
         <v>60</v>
       </c>
-      <c r="D49" s="37" t="s">
+      <c r="D49" s="38" t="s">
         <v>78</v>
       </c>
-      <c r="E49" s="37"/>
+      <c r="E49" s="38"/>
     </row>
     <row r="50" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="10" t="s">
+      <c r="A50" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="B50" s="18"/>
-      <c r="C50" s="45">
+      <c r="B50" s="19"/>
+      <c r="C50" s="43">
         <f>SUM(C45:C49)</f>
         <v>270</v>
       </c>
-      <c r="D50" s="46"/>
-      <c r="E50" s="46"/>
+      <c r="D50" s="44"/>
+      <c r="E50" s="44"/>
     </row>
     <row r="51" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="49" t="s">
+      <c r="A51" s="46" t="s">
         <v>16</v>
       </c>
-      <c r="B51" s="50"/>
-      <c r="C51" s="2">
+      <c r="B51" s="47"/>
+      <c r="C51" s="3">
         <f>MROUND(SUM(C9,C13,C17,C22,C28,C33,C38,C44,C50) /60,0.2)</f>
         <v>27</v>
       </c>
-      <c r="D51" s="3"/>
-      <c r="E51" s="4"/>
+      <c r="D51" s="4"/>
+      <c r="E51" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="14">
@@ -1806,7 +1787,7 @@
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="43" orientation="portrait" r:id="rId8"/>
+  <pageSetup paperSize="9" scale="42" orientation="portrait" r:id="rId8"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Etml_font,Normal"&amp;22ETML&amp;R&amp;G</oddHeader>
     <oddFooter>&amp;L&amp;14&amp;D&amp;R&amp;14Journal</oddFooter>
@@ -1828,6 +1809,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010051C931FEC57CD24D841BB655C8BA0DFF" ma:contentTypeVersion="14" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="f47e485f4ad8d247f3dfedaee1362e95">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3eb094ff-ec8d-44d8-be06-94ad3ec8832a" xmlns:ns3="4356f79f-5386-4bda-9d92-82d8bd7b074e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="da34bf24383b1ce13aa9c82f6b8627bb" ns2:_="" ns3:_="">
     <xsd:import namespace="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
@@ -2040,33 +2030,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
   <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
     <ds:schemaRef ds:uri="4356f79f-5386-4bda-9d92-82d8bd7b074e"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5A40649F-4D7C-4B62-9A51-E0A7D9450EFE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2083,12 +2072,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>